<commit_message>
Exclude SRS_IC from v5.0 Section 3 trial MML (Hold vs tight MUX)
Section 3 now sends Enable/Fix only, with SRS_IC listed in a Hold-this-night table so it is not stacked with CR01 SRS_TIGHT_MULTIPLEXING.

Co-authored-by: Mohammad Selim <miles4482@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MIMO_Deployment_v5.0.xlsx
+++ b/MIMO_Deployment_v5.0.xlsx
@@ -622,7 +622,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="199">
+  <cellXfs count="201">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1121,6 +1121,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -11214,7 +11218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M493"/>
+  <dimension ref="A1:M506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -23862,60 +23866,60 @@
       <c r="M413" s="11" t="n"/>
     </row>
     <row r="414" ht="40" customHeight="1">
-      <c r="A414" s="184" t="n">
+      <c r="A414" s="185" t="n">
         <v>24</v>
       </c>
-      <c r="B414" s="150" t="inlineStr">
+      <c r="B414" s="136" t="inlineStr">
         <is>
           <t>S15-14</t>
         </is>
       </c>
-      <c r="C414" s="40" t="inlineStr">
+      <c r="C414" s="135" t="inlineStr">
         <is>
           <t>Step6</t>
         </is>
       </c>
-      <c r="D414" s="40" t="inlineStr">
+      <c r="D414" s="135" t="inlineStr">
         <is>
           <t>SRS_IC_SW</t>
         </is>
       </c>
-      <c r="E414" s="40" t="inlineStr">
+      <c r="E414" s="135" t="inlineStr">
         <is>
           <t>OFF 564/564</t>
         </is>
       </c>
-      <c r="F414" s="53" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="G414" s="184" t="inlineStr">
+      <c r="F414" s="63" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="G414" s="185" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H414" s="40" t="inlineStr">
+      <c r="H414" s="135" t="inlineStr">
         <is>
           <t>Turbo child off. Tight MUX is in CR01.</t>
         </is>
       </c>
-      <c r="I414" s="40" t="inlineStr">
+      <c r="I414" s="135" t="inlineStr">
         <is>
           <t>Hold this night (do not stack with CR01 tight MUX)</t>
         </is>
       </c>
-      <c r="J414" s="40" t="inlineStr">
+      <c r="J414" s="135" t="inlineStr">
         <is>
           <t>FOFD-061201</t>
         </is>
       </c>
-      <c r="K414" s="150" t="inlineStr">
+      <c r="K414" s="136" t="inlineStr">
         <is>
           <t>S15-14</t>
         </is>
       </c>
-      <c r="L414" s="150" t="inlineStr">
+      <c r="L414" s="136" t="inlineStr">
         <is>
           <t>8. Step6 AHR</t>
         </is>
@@ -24794,7 +24798,7 @@
         </is>
       </c>
       <c r="B432" s="39" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C432" s="40" t="inlineStr">
         <is>
@@ -24819,7 +24823,7 @@
         </is>
       </c>
       <c r="B433" s="64" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C433" s="135" t="inlineStr">
         <is>
@@ -25452,37 +25456,37 @@
       </c>
       <c r="E448" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLSRS: NrDuCellId={NrDuCellId}, SrsDetectionAlgoSwitch=SRS_IC_SW-1;</t>
+          <t>MOD NRDUCELLULPCCONFIG: NrDuCellId={NrDuCellId}, UlPwrCtrlAlgoSwitch=SRS_JOINT_PC_SW-1;</t>
         </is>
       </c>
       <c r="F448" s="42" t="inlineStr">
         <is>
-          <t>NRDUCellSrs</t>
+          <t>NRDUCellUlPcConfig</t>
         </is>
       </c>
       <c r="G448" s="42" t="inlineStr">
         <is>
-          <t>SrsDetectionAlgoSwitch</t>
+          <t>UlPwrCtrlAlgoSwitch</t>
         </is>
       </c>
       <c r="H448" s="42" t="inlineStr">
         <is>
-          <t>SRS_IC OFF 564; BEAM_SPECIFIC_SRS_DENOISE already ON</t>
+          <t>SRS_JOINT_PC OFF 564/564</t>
         </is>
       </c>
       <c r="I448" s="42" t="inlineStr">
         <is>
-          <t>SRS_IC_SW-1</t>
+          <t>SRS_JOINT_PC_SW-1</t>
         </is>
       </c>
       <c r="J448" s="42" t="inlineStr">
         <is>
-          <t>MISSING Turbo child. Watch N.SRS collision / UL SRS quality.</t>
+          <t>Recommended with SRS IC. Live OFF.</t>
         </is>
       </c>
       <c r="K448" s="42" t="inlineStr">
         <is>
-          <t>FOFD-061201 master already ON</t>
+          <t>FOFD-061201</t>
         </is>
       </c>
       <c r="L448" s="197" t="n"/>
@@ -25499,7 +25503,7 @@
       </c>
       <c r="C449" s="60" t="inlineStr">
         <is>
-          <t>AHR Turbo</t>
+          <t>iBeam 1.0</t>
         </is>
       </c>
       <c r="D449" s="53" t="inlineStr">
@@ -25509,37 +25513,37 @@
       </c>
       <c r="E449" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLULPCCONFIG: NrDuCellId={NrDuCellId}, UlPwrCtrlAlgoSwitch=SRS_JOINT_PC_SW-1;</t>
+          <t>MOD NRDUCELLFEATURESW: NrDuCellId={NrDuCellId}, HighPrecisionBeamSwitch=ON;</t>
         </is>
       </c>
       <c r="F449" s="42" t="inlineStr">
         <is>
-          <t>NRDUCellUlPcConfig</t>
+          <t>NRDUCellFeatureSw</t>
         </is>
       </c>
       <c r="G449" s="42" t="inlineStr">
         <is>
-          <t>UlPwrCtrlAlgoSwitch</t>
+          <t>HighPrecisionBeamSwitch</t>
         </is>
       </c>
       <c r="H449" s="42" t="inlineStr">
         <is>
-          <t>SRS_JOINT_PC OFF 564/564</t>
+          <t>OFF 564/564</t>
         </is>
       </c>
       <c r="I449" s="42" t="inlineStr">
         <is>
-          <t>SRS_JOINT_PC_SW-1</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="J449" s="42" t="inlineStr">
         <is>
-          <t>Recommended with SRS IC. Live OFF.</t>
+          <t>MISSING master. iBeam 1.0. Loaded urban 32T.</t>
         </is>
       </c>
       <c r="K449" s="42" t="inlineStr">
         <is>
-          <t>FOFD-061201</t>
+          <t>FOFD-081201 / NR0S00BEAM00 — LST LICENSE</t>
         </is>
       </c>
       <c r="L449" s="197" t="n"/>
@@ -25566,37 +25570,37 @@
       </c>
       <c r="E450" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLFEATURESW: NrDuCellId={NrDuCellId}, HighPrecisionBeamSwitch=ON;</t>
+          <t>MOD NRDUCELLSRSMEAS: NrDuCellId={NrDuCellId}, SrsMeasOptSwitch=SRS_BLIND_IS_MEAS_SW-1;</t>
         </is>
       </c>
       <c r="F450" s="42" t="inlineStr">
         <is>
-          <t>NRDUCellFeatureSw</t>
+          <t>NRDUCellSrsMeas</t>
         </is>
       </c>
       <c r="G450" s="42" t="inlineStr">
         <is>
-          <t>HighPrecisionBeamSwitch</t>
+          <t>SrsMeasOptSwitch</t>
         </is>
       </c>
       <c r="H450" s="42" t="inlineStr">
         <is>
-          <t>OFF 564/564</t>
+          <t>SRS_BLIND_IS_MEAS OFF 564/564</t>
         </is>
       </c>
       <c r="I450" s="42" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>SRS_BLIND_IS_MEAS_SW-1</t>
         </is>
       </c>
       <c r="J450" s="42" t="inlineStr">
         <is>
-          <t>MISSING master. iBeam 1.0. Loaded urban 32T.</t>
+          <t>MISSING. Blind IS for SRS measurement.</t>
         </is>
       </c>
       <c r="K450" s="42" t="inlineStr">
         <is>
-          <t>FOFD-081201 / NR0S00BEAM00 — LST LICENSE</t>
+          <t>FOFD-081201</t>
         </is>
       </c>
       <c r="L450" s="197" t="n"/>
@@ -25623,32 +25627,32 @@
       </c>
       <c r="E451" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLSRSMEAS: NrDuCellId={NrDuCellId}, SrsMeasOptSwitch=SRS_BLIND_IS_MEAS_SW-1;</t>
+          <t>MOD NRDUCELLSRS: NrDuCellId={NrDuCellId}, SrsAlgoSwitch=SRS_TIGHT_MULTIPLEXING_SW-1;</t>
         </is>
       </c>
       <c r="F451" s="42" t="inlineStr">
         <is>
-          <t>NRDUCellSrsMeas</t>
+          <t>NRDUCellSrs</t>
         </is>
       </c>
       <c r="G451" s="42" t="inlineStr">
         <is>
-          <t>SrsMeasOptSwitch</t>
+          <t>SrsAlgoSwitch</t>
         </is>
       </c>
       <c r="H451" s="42" t="inlineStr">
         <is>
-          <t>SRS_BLIND_IS_MEAS OFF 564/564</t>
+          <t>SRS_TIGHT_MULTIPLEXING OFF 564/564</t>
         </is>
       </c>
       <c r="I451" s="42" t="inlineStr">
         <is>
-          <t>SRS_BLIND_IS_MEAS_SW-1</t>
+          <t>SRS_TIGHT_MULTIPLEXING_SW-1</t>
         </is>
       </c>
       <c r="J451" s="42" t="inlineStr">
         <is>
-          <t>MISSING. Blind IS for SRS measurement.</t>
+          <t>MISSING. Do not stack with new SRS_IC the same night.</t>
         </is>
       </c>
       <c r="K451" s="42" t="inlineStr">
@@ -25680,32 +25684,32 @@
       </c>
       <c r="E452" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLSRS: NrDuCellId={NrDuCellId}, SrsAlgoSwitch=SRS_TIGHT_MULTIPLEXING_SW-1;</t>
+          <t>MOD NRDUCELLBEAMALGO: NrDuCellId={NrDuCellId}, ChannelOptAlgoSwitch=BEAM_SELECT_OPT_SW-1;</t>
         </is>
       </c>
       <c r="F452" s="42" t="inlineStr">
         <is>
-          <t>NRDUCellSrs</t>
+          <t>NRDUCellBeamAlgo</t>
         </is>
       </c>
       <c r="G452" s="42" t="inlineStr">
         <is>
-          <t>SrsAlgoSwitch</t>
+          <t>ChannelOptAlgoSwitch</t>
         </is>
       </c>
       <c r="H452" s="42" t="inlineStr">
         <is>
-          <t>SRS_TIGHT_MULTIPLEXING OFF 564/564</t>
+          <t>BEAM_SELECT_OPT OFF 564/564</t>
         </is>
       </c>
       <c r="I452" s="42" t="inlineStr">
         <is>
-          <t>SRS_TIGHT_MULTIPLEXING_SW-1</t>
+          <t>BEAM_SELECT_OPT_SW-1</t>
         </is>
       </c>
       <c r="J452" s="42" t="inlineStr">
         <is>
-          <t>MISSING. Do not stack with new SRS_IC the same night.</t>
+          <t>MISSING. Beam selection optimization.</t>
         </is>
       </c>
       <c r="K452" s="42" t="inlineStr">
@@ -25737,32 +25741,32 @@
       </c>
       <c r="E453" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLBEAMALGO: NrDuCellId={NrDuCellId}, ChannelOptAlgoSwitch=BEAM_SELECT_OPT_SW-1;</t>
+          <t>MOD NRDUCELLDLMIMO: NrDuCellId={NrDuCellId}, DLMuMimoSchSupplementSw=DL_MU_PRECISE_SCH_SW-1;</t>
         </is>
       </c>
       <c r="F453" s="42" t="inlineStr">
         <is>
-          <t>NRDUCellBeamAlgo</t>
+          <t>NRDUCellDlMimo</t>
         </is>
       </c>
       <c r="G453" s="42" t="inlineStr">
         <is>
-          <t>ChannelOptAlgoSwitch</t>
+          <t>DLMuMimoSchSupplementSw</t>
         </is>
       </c>
       <c r="H453" s="42" t="inlineStr">
         <is>
-          <t>BEAM_SELECT_OPT OFF 564/564</t>
+          <t>DL_MU_PRECISE_SCH OFF 564/564</t>
         </is>
       </c>
       <c r="I453" s="42" t="inlineStr">
         <is>
-          <t>BEAM_SELECT_OPT_SW-1</t>
+          <t>DL_MU_PRECISE_SCH_SW-1</t>
         </is>
       </c>
       <c r="J453" s="42" t="inlineStr">
         <is>
-          <t>MISSING. Beam selection optimization.</t>
+          <t>MISSING. DL MU precise scheduling — MU efficiency under interference.</t>
         </is>
       </c>
       <c r="K453" s="42" t="inlineStr">
@@ -25794,7 +25798,7 @@
       </c>
       <c r="E454" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLDLMIMO: NrDuCellId={NrDuCellId}, DLMuMimoSchSupplementSw=DL_MU_PRECISE_SCH_SW-1;</t>
+          <t>MOD NRDUCELLDLMIMO: NrDuCellId={NrDuCellId}, DLMuMimoSchSupplementSw=DL_MU_ANTI_INTRF_SCH_SW-1;</t>
         </is>
       </c>
       <c r="F454" s="42" t="inlineStr">
@@ -25809,17 +25813,17 @@
       </c>
       <c r="H454" s="42" t="inlineStr">
         <is>
-          <t>DL_MU_PRECISE_SCH OFF 564/564</t>
+          <t>DL_MU_ANTI_INTRF_SCH OFF 564/564</t>
         </is>
       </c>
       <c r="I454" s="42" t="inlineStr">
         <is>
-          <t>DL_MU_PRECISE_SCH_SW-1</t>
+          <t>DL_MU_ANTI_INTRF_SCH_SW-1</t>
         </is>
       </c>
       <c r="J454" s="42" t="inlineStr">
         <is>
-          <t>MISSING. DL MU precise scheduling — MU efficiency under interference.</t>
+          <t>MISSING. DL MU anti-interference scheduling.</t>
         </is>
       </c>
       <c r="K454" s="42" t="inlineStr">
@@ -25851,32 +25855,32 @@
       </c>
       <c r="E455" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLDLMIMO: NrDuCellId={NrDuCellId}, DLMuMimoSchSupplementSw=DL_MU_ANTI_INTRF_SCH_SW-1;</t>
+          <t>MOD NRDUCELLDLSCH: NrDuCellId={NrDuCellId}, DlSchAlgoSwitch=DL_BWP_HYBRID_INTRF_RANDOM_SW-1;</t>
         </is>
       </c>
       <c r="F455" s="42" t="inlineStr">
         <is>
-          <t>NRDUCellDlMimo</t>
+          <t>NRDUCellDlSch</t>
         </is>
       </c>
       <c r="G455" s="42" t="inlineStr">
         <is>
-          <t>DLMuMimoSchSupplementSw</t>
+          <t>DlSchAlgoSwitch</t>
         </is>
       </c>
       <c r="H455" s="42" t="inlineStr">
         <is>
-          <t>DL_MU_ANTI_INTRF_SCH OFF 564/564</t>
+          <t>DL_BWP_HYBRID_INTRF_RANDOM OFF 564/564</t>
         </is>
       </c>
       <c r="I455" s="42" t="inlineStr">
         <is>
-          <t>DL_MU_ANTI_INTRF_SCH_SW-1</t>
+          <t>DL_BWP_HYBRID_INTRF_RANDOM_SW-1</t>
         </is>
       </c>
       <c r="J455" s="42" t="inlineStr">
         <is>
-          <t>MISSING. DL MU anti-interference scheduling.</t>
+          <t>MISSING. DL multi-BWP interference randomization.</t>
         </is>
       </c>
       <c r="K455" s="42" t="inlineStr">
@@ -25908,7 +25912,7 @@
       </c>
       <c r="E456" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLDLSCH: NrDuCellId={NrDuCellId}, DlSchAlgoSwitch=DL_BWP_HYBRID_INTRF_RANDOM_SW-1;</t>
+          <t>MOD NRDUCELLDLSCH: NrDuCellId={NrDuCellId}, DlSchAlgoSwitch=TAIL_PKT_MCS_OPT_SW-1;</t>
         </is>
       </c>
       <c r="F456" s="42" t="inlineStr">
@@ -25923,17 +25927,17 @@
       </c>
       <c r="H456" s="42" t="inlineStr">
         <is>
-          <t>DL_BWP_HYBRID_INTRF_RANDOM OFF 564/564</t>
+          <t>TAIL_PKT_MCS_OPT OFF 564/564 (PDSCH TAIL_PKT_SCH_OPT already ON — different bit)</t>
         </is>
       </c>
       <c r="I456" s="42" t="inlineStr">
         <is>
-          <t>DL_BWP_HYBRID_INTRF_RANDOM_SW-1</t>
+          <t>TAIL_PKT_MCS_OPT_SW-1</t>
         </is>
       </c>
       <c r="J456" s="42" t="inlineStr">
         <is>
-          <t>MISSING. DL multi-BWP interference randomization.</t>
+          <t>MISSING. Tail-packet MCS opt. Complements already-ON TAIL_PKT_SCH_OPT.</t>
         </is>
       </c>
       <c r="K456" s="42" t="inlineStr">
@@ -25965,7 +25969,7 @@
       </c>
       <c r="E457" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLDLSCH: NrDuCellId={NrDuCellId}, DlSchAlgoSwitch=TAIL_PKT_MCS_OPT_SW-1;</t>
+          <t>MOD NRDUCELLDLSCH: NrDuCellId={NrDuCellId}, DlSchAlgoSwitch=RES_BASED_DL_ADAPT_SCH_SW-1;</t>
         </is>
       </c>
       <c r="F457" s="42" t="inlineStr">
@@ -25980,17 +25984,17 @@
       </c>
       <c r="H457" s="42" t="inlineStr">
         <is>
-          <t>TAIL_PKT_MCS_OPT OFF 564/564 (PDSCH TAIL_PKT_SCH_OPT already ON — different bit)</t>
+          <t>RES_BASED_DL_ADAPT_SCH OFF 564/564</t>
         </is>
       </c>
       <c r="I457" s="42" t="inlineStr">
         <is>
-          <t>TAIL_PKT_MCS_OPT_SW-1</t>
+          <t>RES_BASED_DL_ADAPT_SCH_SW-1</t>
         </is>
       </c>
       <c r="J457" s="42" t="inlineStr">
         <is>
-          <t>MISSING. Tail-packet MCS opt. Complements already-ON TAIL_PKT_SCH_OPT.</t>
+          <t>MISSING. Resource-based adaptive DL scheduling.</t>
         </is>
       </c>
       <c r="K457" s="42" t="inlineStr">
@@ -26022,7 +26026,7 @@
       </c>
       <c r="E458" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLDLSCH: NrDuCellId={NrDuCellId}, DlSchAlgoSwitch=RES_BASED_DL_ADAPT_SCH_SW-1;</t>
+          <t>MOD NRDUCELLDLSCH: NrDuCellId={NrDuCellId}, DlSchAlgoSwitch=DL_RLC_STAT_RPT_MERGE_SCH_SW-1;</t>
         </is>
       </c>
       <c r="F458" s="42" t="inlineStr">
@@ -26037,17 +26041,17 @@
       </c>
       <c r="H458" s="42" t="inlineStr">
         <is>
-          <t>RES_BASED_DL_ADAPT_SCH OFF 564/564</t>
+          <t>DL_RLC_STAT_RPT_MERGE_SCH OFF 564/564</t>
         </is>
       </c>
       <c r="I458" s="42" t="inlineStr">
         <is>
-          <t>RES_BASED_DL_ADAPT_SCH_SW-1</t>
+          <t>DL_RLC_STAT_RPT_MERGE_SCH_SW-1</t>
         </is>
       </c>
       <c r="J458" s="42" t="inlineStr">
         <is>
-          <t>MISSING. Resource-based adaptive DL scheduling.</t>
+          <t>MISSING. Merged DL RLC status-report scheduling.</t>
         </is>
       </c>
       <c r="K458" s="42" t="inlineStr">
@@ -26079,32 +26083,32 @@
       </c>
       <c r="E459" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLDLSCH: NrDuCellId={NrDuCellId}, DlSchAlgoSwitch=DL_RLC_STAT_RPT_MERGE_SCH_SW-1;</t>
+          <t>MOD NRDUCELLPDCCH: NrDuCellId={NrDuCellId}, PdcchAlgoSwitch=PDCCH_AGG_LVL_COMPR_SW-1;</t>
         </is>
       </c>
       <c r="F459" s="42" t="inlineStr">
         <is>
-          <t>NRDUCellDlSch</t>
+          <t>NRDUCellPdcch</t>
         </is>
       </c>
       <c r="G459" s="42" t="inlineStr">
         <is>
-          <t>DlSchAlgoSwitch</t>
+          <t>PdcchAlgoSwitch</t>
         </is>
       </c>
       <c r="H459" s="42" t="inlineStr">
         <is>
-          <t>DL_RLC_STAT_RPT_MERGE_SCH OFF 564/564</t>
+          <t>PDCCH_AGG_LVL_COMPR OFF 564 (threshold already 60)</t>
         </is>
       </c>
       <c r="I459" s="42" t="inlineStr">
         <is>
-          <t>DL_RLC_STAT_RPT_MERGE_SCH_SW-1</t>
+          <t>PDCCH_AGG_LVL_COMPR_SW-1</t>
         </is>
       </c>
       <c r="J459" s="42" t="inlineStr">
         <is>
-          <t>MISSING. Merged DL RLC status-report scheduling.</t>
+          <t>MISSING. PDCCH aggregation-level compression. Threshold already staged at 60.</t>
         </is>
       </c>
       <c r="K459" s="42" t="inlineStr">
@@ -26126,7 +26130,7 @@
       </c>
       <c r="C460" s="60" t="inlineStr">
         <is>
-          <t>iBeam 1.0</t>
+          <t>UL Boosting 1.0</t>
         </is>
       </c>
       <c r="D460" s="53" t="inlineStr">
@@ -26136,37 +26140,37 @@
       </c>
       <c r="E460" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLPDCCH: NrDuCellId={NrDuCellId}, PdcchAlgoSwitch=PDCCH_AGG_LVL_COMPR_SW-1;</t>
+          <t>MOD NRDUCELLFEATURESW: NrDuCellId={NrDuCellId}, MimoFeatureSwitch=UL_LOW_NOISE_SW-1;</t>
         </is>
       </c>
       <c r="F460" s="42" t="inlineStr">
         <is>
-          <t>NRDUCellPdcch</t>
+          <t>NRDUCellFeatureSw</t>
         </is>
       </c>
       <c r="G460" s="42" t="inlineStr">
         <is>
-          <t>PdcchAlgoSwitch</t>
+          <t>MimoFeatureSwitch</t>
         </is>
       </c>
       <c r="H460" s="42" t="inlineStr">
         <is>
-          <t>PDCCH_AGG_LVL_COMPR OFF 564 (threshold already 60)</t>
+          <t>UL_LOW_NOISE_SW OFF 564/564</t>
         </is>
       </c>
       <c r="I460" s="42" t="inlineStr">
         <is>
-          <t>PDCCH_AGG_LVL_COMPR_SW-1</t>
+          <t>UL_LOW_NOISE_SW-1</t>
         </is>
       </c>
       <c r="J460" s="42" t="inlineStr">
         <is>
-          <t>MISSING. PDCCH aggregation-level compression. Threshold already staged at 60.</t>
+          <t>MISSING master. Uplink Boosting 1.0.</t>
         </is>
       </c>
       <c r="K460" s="42" t="inlineStr">
         <is>
-          <t>FOFD-081201</t>
+          <t>FOFD-091201 / NR0S00UAHR00 — LST LICENSE</t>
         </is>
       </c>
       <c r="L460" s="197" t="n"/>
@@ -26193,37 +26197,37 @@
       </c>
       <c r="E461" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLFEATURESW: NrDuCellId={NrDuCellId}, MimoFeatureSwitch=UL_LOW_NOISE_SW-1;</t>
+          <t>MOD NRDUCELLULMIMO: NrDuCellId={NrDuCellId}, UlMuMimoAlgoSwitch=UL_MU_GRP_PAIR_SW-1;</t>
         </is>
       </c>
       <c r="F461" s="42" t="inlineStr">
         <is>
-          <t>NRDUCellFeatureSw</t>
+          <t>NRDUCellUlMimo</t>
         </is>
       </c>
       <c r="G461" s="42" t="inlineStr">
         <is>
-          <t>MimoFeatureSwitch</t>
+          <t>UlMuMimoAlgoSwitch</t>
         </is>
       </c>
       <c r="H461" s="42" t="inlineStr">
         <is>
-          <t>UL_LOW_NOISE_SW OFF 564/564</t>
+          <t>UL_MU_GRP_PAIR OFF 564/564</t>
         </is>
       </c>
       <c r="I461" s="42" t="inlineStr">
         <is>
-          <t>UL_LOW_NOISE_SW-1</t>
+          <t>UL_MU_GRP_PAIR_SW-1</t>
         </is>
       </c>
       <c r="J461" s="42" t="inlineStr">
         <is>
-          <t>MISSING master. Uplink Boosting 1.0.</t>
+          <t>MISSING. UL MU grouping/pairing.</t>
         </is>
       </c>
       <c r="K461" s="42" t="inlineStr">
         <is>
-          <t>FOFD-091201 / NR0S00UAHR00 — LST LICENSE</t>
+          <t>FOFD-091201</t>
         </is>
       </c>
       <c r="L461" s="197" t="n"/>
@@ -26250,7 +26254,7 @@
       </c>
       <c r="E462" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLULMIMO: NrDuCellId={NrDuCellId}, UlMuMimoAlgoSwitch=UL_MU_GRP_PAIR_SW-1;</t>
+          <t>MOD NRDUCELLULMIMO: NrDuCellId={NrDuCellId}, UlMuMimoAlgoSwitch=DIFF_WAVEFORM_PAIR_SW-1;</t>
         </is>
       </c>
       <c r="F462" s="42" t="inlineStr">
@@ -26265,17 +26269,17 @@
       </c>
       <c r="H462" s="42" t="inlineStr">
         <is>
-          <t>UL_MU_GRP_PAIR OFF 564/564</t>
+          <t>DIFF_WAVEFORM_PAIR OFF 564/564</t>
         </is>
       </c>
       <c r="I462" s="42" t="inlineStr">
         <is>
-          <t>UL_MU_GRP_PAIR_SW-1</t>
+          <t>DIFF_WAVEFORM_PAIR_SW-1</t>
         </is>
       </c>
       <c r="J462" s="42" t="inlineStr">
         <is>
-          <t>MISSING. UL MU grouping/pairing.</t>
+          <t>MISSING. Mixed-waveform UL MU pairing.</t>
         </is>
       </c>
       <c r="K462" s="42" t="inlineStr">
@@ -26307,7 +26311,7 @@
       </c>
       <c r="E463" s="39" t="inlineStr">
         <is>
-          <t>MOD NRDUCELLULMIMO: NrDuCellId={NrDuCellId}, UlMuMimoAlgoSwitch=DIFF_WAVEFORM_PAIR_SW-1;</t>
+          <t>MOD NRDUCELLULMIMO: NrDuCellId={NrDuCellId}, UlMuMimoAlgoSwitch=UL_CORR_ACCELERATION_SW-1;</t>
         </is>
       </c>
       <c r="F463" s="42" t="inlineStr">
@@ -26322,17 +26326,17 @@
       </c>
       <c r="H463" s="42" t="inlineStr">
         <is>
-          <t>DIFF_WAVEFORM_PAIR OFF 564/564</t>
+          <t>UL_CORR_ACCELERATION OFF 564/564</t>
         </is>
       </c>
       <c r="I463" s="42" t="inlineStr">
         <is>
-          <t>DIFF_WAVEFORM_PAIR_SW-1</t>
+          <t>UL_CORR_ACCELERATION_SW-1</t>
         </is>
       </c>
       <c r="J463" s="42" t="inlineStr">
         <is>
-          <t>MISSING. Mixed-waveform UL MU pairing.</t>
+          <t>MISSING. UL correlation-acceleration pairing.</t>
         </is>
       </c>
       <c r="K463" s="42" t="inlineStr">
@@ -26343,66 +26347,457 @@
       <c r="L463" s="197" t="n"/>
       <c r="M463" s="197" t="n"/>
     </row>
-    <row r="464" ht="40" customHeight="1">
-      <c r="A464" s="59" t="n">
-        <v>24</v>
-      </c>
-      <c r="B464" s="59" t="inlineStr">
-        <is>
-          <t>TDD</t>
-        </is>
-      </c>
-      <c r="C464" s="60" t="inlineStr">
-        <is>
-          <t>UL Boosting 1.0</t>
-        </is>
-      </c>
-      <c r="D464" s="53" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="E464" s="39" t="inlineStr">
-        <is>
-          <t>MOD NRDUCELLULMIMO: NrDuCellId={NrDuCellId}, UlMuMimoAlgoSwitch=UL_CORR_ACCELERATION_SW-1;</t>
-        </is>
-      </c>
-      <c r="F464" s="42" t="inlineStr">
-        <is>
-          <t>NRDUCellUlMimo</t>
-        </is>
-      </c>
-      <c r="G464" s="42" t="inlineStr">
-        <is>
-          <t>UlMuMimoAlgoSwitch</t>
-        </is>
-      </c>
-      <c r="H464" s="42" t="inlineStr">
-        <is>
-          <t>UL_CORR_ACCELERATION OFF 564/564</t>
-        </is>
-      </c>
-      <c r="I464" s="42" t="inlineStr">
-        <is>
-          <t>UL_CORR_ACCELERATION_SW-1</t>
-        </is>
-      </c>
-      <c r="J464" s="42" t="inlineStr">
-        <is>
-          <t>MISSING. UL correlation-acceleration pairing.</t>
-        </is>
-      </c>
-      <c r="K464" s="42" t="inlineStr">
-        <is>
-          <t>FOFD-091201</t>
-        </is>
-      </c>
-      <c r="L464" s="197" t="n"/>
-      <c r="M464" s="197" t="n"/>
-    </row>
-    <row r="465" ht="8" customHeight="1"/>
-    <row r="466" ht="72" customHeight="1">
-      <c r="A466" s="13" t="inlineStr">
+    <row r="464" ht="8" customHeight="1"/>
+    <row r="465" ht="20" customHeight="1">
+      <c r="A465" s="198" t="inlineStr">
+        <is>
+          <t>Still OFF — Hold this night (not in the trial MML above)</t>
+        </is>
+      </c>
+      <c r="B465" s="199" t="n"/>
+      <c r="C465" s="199" t="n"/>
+      <c r="D465" s="199" t="n"/>
+      <c r="E465" s="199" t="n"/>
+      <c r="F465" s="199" t="n"/>
+      <c r="G465" s="199" t="n"/>
+      <c r="H465" s="199" t="n"/>
+      <c r="I465" s="199" t="n"/>
+      <c r="J465" s="199" t="n"/>
+      <c r="K465" s="199" t="n"/>
+      <c r="L465" s="199" t="n"/>
+      <c r="M465" s="199" t="n"/>
+    </row>
+    <row r="466" ht="28" customHeight="1">
+      <c r="A466" s="16" t="inlineStr">
+        <is>
+          <t>These are not enabled on the cluster either, but they are not the Section 3 send list. SRS_IC stays Hold while CR01 SRS_TIGHT_MULTIPLEXING is ON. PMI/open-loop stay Hold while SRS weight is ON.</t>
+        </is>
+      </c>
+      <c r="B466" s="17" t="n"/>
+      <c r="C466" s="17" t="n"/>
+      <c r="D466" s="17" t="n"/>
+      <c r="E466" s="17" t="n"/>
+      <c r="F466" s="17" t="n"/>
+      <c r="G466" s="17" t="n"/>
+      <c r="H466" s="17" t="n"/>
+      <c r="I466" s="17" t="n"/>
+      <c r="J466" s="17" t="n"/>
+      <c r="K466" s="17" t="n"/>
+      <c r="L466" s="17" t="n"/>
+      <c r="M466" s="17" t="n"/>
+    </row>
+    <row r="467" ht="22" customHeight="1">
+      <c r="A467" s="7" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B467" s="7" t="inlineStr">
+        <is>
+          <t>Suggestion</t>
+        </is>
+      </c>
+      <c r="C467" s="7" t="inlineStr">
+        <is>
+          <t>Parameter / switch</t>
+        </is>
+      </c>
+      <c r="D467" s="7" t="inlineStr">
+        <is>
+          <t>Dump status</t>
+        </is>
+      </c>
+      <c r="E467" s="7" t="inlineStr">
+        <is>
+          <t>Why Hold</t>
+        </is>
+      </c>
+      <c r="F467" s="7" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+      <c r="G467" s="7" t="inlineStr"/>
+      <c r="H467" s="7" t="inlineStr"/>
+      <c r="I467" s="7" t="inlineStr"/>
+      <c r="J467" s="7" t="inlineStr"/>
+      <c r="K467" s="7" t="inlineStr"/>
+      <c r="L467" s="7" t="inlineStr"/>
+      <c r="M467" s="7" t="inlineStr"/>
+    </row>
+    <row r="468" ht="28" customHeight="1">
+      <c r="A468" s="185" t="n">
+        <v>1</v>
+      </c>
+      <c r="B468" s="136" t="inlineStr">
+        <is>
+          <t>S15-02</t>
+        </is>
+      </c>
+      <c r="C468" s="135" t="inlineStr">
+        <is>
+          <t>PMI_WEIGHT_OPT_SW</t>
+        </is>
+      </c>
+      <c r="D468" s="63" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="E468" s="135" t="inlineStr">
+        <is>
+          <t>Missing vs FPD but mix with SRS tonight.</t>
+        </is>
+      </c>
+      <c r="F468" s="135" t="inlineStr">
+        <is>
+          <t>Hold first night</t>
+        </is>
+      </c>
+      <c r="G468" s="10" t="n"/>
+      <c r="H468" s="10" t="n"/>
+      <c r="I468" s="10" t="n"/>
+      <c r="J468" s="10" t="n"/>
+      <c r="K468" s="10" t="n"/>
+      <c r="L468" s="10" t="n"/>
+      <c r="M468" s="11" t="n"/>
+    </row>
+    <row r="469" ht="28" customHeight="1">
+      <c r="A469" s="185" t="n">
+        <v>2</v>
+      </c>
+      <c r="B469" s="136" t="inlineStr">
+        <is>
+          <t>S15-02</t>
+        </is>
+      </c>
+      <c r="C469" s="135" t="inlineStr">
+        <is>
+          <t>OPEN_LOOP_WEIGHT_OPT_SW</t>
+        </is>
+      </c>
+      <c r="D469" s="63" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="E469" s="135" t="inlineStr">
+        <is>
+          <t>Same mix rule.</t>
+        </is>
+      </c>
+      <c r="F469" s="135" t="inlineStr">
+        <is>
+          <t>Hold first night</t>
+        </is>
+      </c>
+      <c r="G469" s="10" t="n"/>
+      <c r="H469" s="10" t="n"/>
+      <c r="I469" s="10" t="n"/>
+      <c r="J469" s="10" t="n"/>
+      <c r="K469" s="10" t="n"/>
+      <c r="L469" s="10" t="n"/>
+      <c r="M469" s="11" t="n"/>
+    </row>
+    <row r="470" ht="28" customHeight="1">
+      <c r="A470" s="185" t="n">
+        <v>3</v>
+      </c>
+      <c r="B470" s="136" t="inlineStr">
+        <is>
+          <t>S15-09</t>
+        </is>
+      </c>
+      <c r="C470" s="135" t="inlineStr">
+        <is>
+          <t>MMIMO_MULTILAYER_ENHANCE / PAIRING_PREFERRED / MU_RANK_BOOSTING / SRS_MEAS_ACCELERATING</t>
+        </is>
+      </c>
+      <c r="D470" s="63" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="E470" s="135" t="inlineStr">
+        <is>
+          <t>Quota LAYER_16 unused.</t>
+        </is>
+      </c>
+      <c r="F470" s="135" t="inlineStr">
+        <is>
+          <t>Next CR after iBeam 1.0 green</t>
+        </is>
+      </c>
+      <c r="G470" s="10" t="n"/>
+      <c r="H470" s="10" t="n"/>
+      <c r="I470" s="10" t="n"/>
+      <c r="J470" s="10" t="n"/>
+      <c r="K470" s="10" t="n"/>
+      <c r="L470" s="10" t="n"/>
+      <c r="M470" s="11" t="n"/>
+    </row>
+    <row r="471" ht="28" customHeight="1">
+      <c r="A471" s="185" t="n">
+        <v>4</v>
+      </c>
+      <c r="B471" s="136" t="inlineStr">
+        <is>
+          <t>S15-10</t>
+        </is>
+      </c>
+      <c r="C471" s="135" t="inlineStr">
+        <is>
+          <t>UL MULTILAYER_DEMOD_ENH / FLEX_PAIR / RES_BASED_ULSCH</t>
+        </is>
+      </c>
+      <c r="D471" s="63" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="E471" s="135" t="inlineStr">
+        <is>
+          <t>UL multilayer not started.</t>
+        </is>
+      </c>
+      <c r="F471" s="135" t="inlineStr">
+        <is>
+          <t>After DL multilayer</t>
+        </is>
+      </c>
+      <c r="G471" s="10" t="n"/>
+      <c r="H471" s="10" t="n"/>
+      <c r="I471" s="10" t="n"/>
+      <c r="J471" s="10" t="n"/>
+      <c r="K471" s="10" t="n"/>
+      <c r="L471" s="10" t="n"/>
+      <c r="M471" s="11" t="n"/>
+    </row>
+    <row r="472" ht="28" customHeight="1">
+      <c r="A472" s="185" t="n">
+        <v>5</v>
+      </c>
+      <c r="B472" s="136" t="inlineStr">
+        <is>
+          <t>S15-14</t>
+        </is>
+      </c>
+      <c r="C472" s="135" t="inlineStr">
+        <is>
+          <t>SRS_IC_SW</t>
+        </is>
+      </c>
+      <c r="D472" s="63" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="E472" s="135" t="inlineStr">
+        <is>
+          <t>Turbo child off. Tight MUX is in CR01.</t>
+        </is>
+      </c>
+      <c r="F472" s="135" t="inlineStr">
+        <is>
+          <t>Hold this night (do not stack with CR01 tight MUX)</t>
+        </is>
+      </c>
+      <c r="G472" s="10" t="n"/>
+      <c r="H472" s="10" t="n"/>
+      <c r="I472" s="10" t="n"/>
+      <c r="J472" s="10" t="n"/>
+      <c r="K472" s="10" t="n"/>
+      <c r="L472" s="10" t="n"/>
+      <c r="M472" s="11" t="n"/>
+    </row>
+    <row r="473" ht="28" customHeight="1">
+      <c r="A473" s="185" t="n">
+        <v>6</v>
+      </c>
+      <c r="B473" s="136" t="inlineStr">
+        <is>
+          <t>S15-15</t>
+        </is>
+      </c>
+      <c r="C473" s="135" t="inlineStr">
+        <is>
+          <t>AHR_CAPC_UPGRADE_PHASE2 + PDCCH_MULTI_DIM_JOINT_SCH</t>
+        </is>
+      </c>
+      <c r="D473" s="63" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="E473" s="135" t="inlineStr">
+        <is>
+          <t>Capacity wave never started.</t>
+        </is>
+      </c>
+      <c r="F473" s="135" t="inlineStr">
+        <is>
+          <t>After Turbo SRS-IC + iBeam 1.0 green</t>
+        </is>
+      </c>
+      <c r="G473" s="10" t="n"/>
+      <c r="H473" s="10" t="n"/>
+      <c r="I473" s="10" t="n"/>
+      <c r="J473" s="10" t="n"/>
+      <c r="K473" s="10" t="n"/>
+      <c r="L473" s="10" t="n"/>
+      <c r="M473" s="11" t="n"/>
+    </row>
+    <row r="474" ht="28" customHeight="1">
+      <c r="A474" s="185" t="n">
+        <v>7</v>
+      </c>
+      <c r="B474" s="136" t="inlineStr">
+        <is>
+          <t>S15-17</t>
+        </is>
+      </c>
+      <c r="C474" s="135" t="inlineStr">
+        <is>
+          <t>HighPrecisionBeamPhase2Sw / DL_ROBUST_WEIGHT</t>
+        </is>
+      </c>
+      <c r="D474" s="63" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="E474" s="135" t="inlineStr">
+        <is>
+          <t>Correctly not started — 1.0 missing on cluster.</t>
+        </is>
+      </c>
+      <c r="F474" s="135" t="inlineStr">
+        <is>
+          <t>Do not enable now</t>
+        </is>
+      </c>
+      <c r="G474" s="10" t="n"/>
+      <c r="H474" s="10" t="n"/>
+      <c r="I474" s="10" t="n"/>
+      <c r="J474" s="10" t="n"/>
+      <c r="K474" s="10" t="n"/>
+      <c r="L474" s="10" t="n"/>
+      <c r="M474" s="11" t="n"/>
+    </row>
+    <row r="475" ht="28" customHeight="1">
+      <c r="A475" s="185" t="n">
+        <v>8</v>
+      </c>
+      <c r="B475" s="136" t="inlineStr">
+        <is>
+          <t>S15-18</t>
+        </is>
+      </c>
+      <c r="C475" s="135" t="inlineStr">
+        <is>
+          <t>HighPrecisionBeamPhase3Sw / DL_SELF_FUSION_WEIGHT</t>
+        </is>
+      </c>
+      <c r="D475" s="63" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="E475" s="135" t="inlineStr">
+        <is>
+          <t>Last wave.</t>
+        </is>
+      </c>
+      <c r="F475" s="135" t="inlineStr">
+        <is>
+          <t>After 2.0 green</t>
+        </is>
+      </c>
+      <c r="G475" s="10" t="n"/>
+      <c r="H475" s="10" t="n"/>
+      <c r="I475" s="10" t="n"/>
+      <c r="J475" s="10" t="n"/>
+      <c r="K475" s="10" t="n"/>
+      <c r="L475" s="10" t="n"/>
+      <c r="M475" s="11" t="n"/>
+    </row>
+    <row r="476" ht="28" customHeight="1">
+      <c r="A476" s="185" t="n">
+        <v>9</v>
+      </c>
+      <c r="B476" s="136" t="inlineStr">
+        <is>
+          <t>S15-20</t>
+        </is>
+      </c>
+      <c r="C476" s="135" t="inlineStr">
+        <is>
+          <t>UL_LOW_NOISE_PHASE2_SW</t>
+        </is>
+      </c>
+      <c r="D476" s="63" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="E476" s="135" t="inlineStr">
+        <is>
+          <t>After 1.0 KPI-green + sync.</t>
+        </is>
+      </c>
+      <c r="F476" s="135" t="inlineStr">
+        <is>
+          <t>Not this CR</t>
+        </is>
+      </c>
+      <c r="G476" s="10" t="n"/>
+      <c r="H476" s="10" t="n"/>
+      <c r="I476" s="10" t="n"/>
+      <c r="J476" s="10" t="n"/>
+      <c r="K476" s="10" t="n"/>
+      <c r="L476" s="10" t="n"/>
+      <c r="M476" s="11" t="n"/>
+    </row>
+    <row r="477" ht="28" customHeight="1">
+      <c r="A477" s="185" t="n">
+        <v>10</v>
+      </c>
+      <c r="B477" s="136" t="inlineStr">
+        <is>
+          <t>S15-25</t>
+        </is>
+      </c>
+      <c r="C477" s="135" t="inlineStr">
+        <is>
+          <t>FREQ_SEL_SCH / LOAD_BASED_DL_EXP_SCH / SMART_SCH / HIGH_CAPACITY_EXP</t>
+        </is>
+      </c>
+      <c r="D477" s="63" t="inlineStr">
+        <is>
+          <t>Hold</t>
+        </is>
+      </c>
+      <c r="E477" s="135" t="inlineStr">
+        <is>
+          <t>Beyond iBeam 1.0 minimum.</t>
+        </is>
+      </c>
+      <c r="F477" s="135" t="inlineStr">
+        <is>
+          <t>After CSI/iBeam 1.0 green; license+TAC for smart/high-cap</t>
+        </is>
+      </c>
+      <c r="G477" s="10" t="n"/>
+      <c r="H477" s="10" t="n"/>
+      <c r="I477" s="10" t="n"/>
+      <c r="J477" s="10" t="n"/>
+      <c r="K477" s="10" t="n"/>
+      <c r="L477" s="10" t="n"/>
+      <c r="M477" s="11" t="n"/>
+    </row>
+    <row r="478" ht="8" customHeight="1"/>
+    <row r="479" ht="72" customHeight="1">
+      <c r="A479" s="13" t="inlineStr">
         <is>
           <t>•  Cluster still OFF after CR01: same Enable list on the remaining 32T (not the 10 trial gNB).
 •  Hold (not in this proposal): PMI_WEIGHT_OPT / OPEN_LOOP_WEIGHT_OPT; SRS_IC while tight MUX is ON; multilayer; AHR CU 2.0; iBeam 2.0/3.0; freq-sel/smart sch; Boosting 2.0.
@@ -26410,1031 +26805,1031 @@
 •  Rollback: set the enabled bit back to 0 / HighPrecisionBeamSwitch=OFF / UL_LOW_NOISE_SW-0. Do not touch SU/MU/AHR Phase1+Turbo/LAYER_16.</t>
         </is>
       </c>
-      <c r="B466" s="14" t="n"/>
-      <c r="C466" s="14" t="n"/>
-      <c r="D466" s="14" t="n"/>
-      <c r="E466" s="14" t="n"/>
-      <c r="F466" s="14" t="n"/>
-      <c r="G466" s="14" t="n"/>
-      <c r="H466" s="14" t="n"/>
-      <c r="I466" s="14" t="n"/>
-      <c r="J466" s="14" t="n"/>
-      <c r="K466" s="14" t="n"/>
-      <c r="L466" s="14" t="n"/>
-      <c r="M466" s="14" t="n"/>
-    </row>
-    <row r="467" ht="22" customHeight="1">
-      <c r="A467" s="198" t="inlineStr">
+      <c r="B479" s="14" t="n"/>
+      <c r="C479" s="14" t="n"/>
+      <c r="D479" s="14" t="n"/>
+      <c r="E479" s="14" t="n"/>
+      <c r="F479" s="14" t="n"/>
+      <c r="G479" s="14" t="n"/>
+      <c r="H479" s="14" t="n"/>
+      <c r="I479" s="14" t="n"/>
+      <c r="J479" s="14" t="n"/>
+      <c r="K479" s="14" t="n"/>
+      <c r="L479" s="14" t="n"/>
+      <c r="M479" s="14" t="n"/>
+    </row>
+    <row r="480" ht="22" customHeight="1">
+      <c r="A480" s="200" t="inlineStr">
         <is>
           <t>Section 4.  Performance counter and Monitoring KPI</t>
         </is>
       </c>
-      <c r="B467" s="133" t="n"/>
-      <c r="C467" s="133" t="n"/>
-      <c r="D467" s="133" t="n"/>
-      <c r="E467" s="133" t="n"/>
-      <c r="F467" s="133" t="n"/>
-      <c r="G467" s="133" t="n"/>
-      <c r="H467" s="133" t="n"/>
-      <c r="I467" s="133" t="n"/>
-      <c r="J467" s="133" t="n"/>
-      <c r="K467" s="133" t="n"/>
-      <c r="L467" s="133" t="n"/>
-      <c r="M467" s="133" t="n"/>
-    </row>
-    <row r="468" ht="28" customHeight="1">
-      <c r="A468" s="16" t="inlineStr">
+      <c r="B480" s="133" t="n"/>
+      <c r="C480" s="133" t="n"/>
+      <c r="D480" s="133" t="n"/>
+      <c r="E480" s="133" t="n"/>
+      <c r="F480" s="133" t="n"/>
+      <c r="G480" s="133" t="n"/>
+      <c r="H480" s="133" t="n"/>
+      <c r="I480" s="133" t="n"/>
+      <c r="J480" s="133" t="n"/>
+      <c r="K480" s="133" t="n"/>
+      <c r="L480" s="133" t="n"/>
+      <c r="M480" s="133" t="n"/>
+    </row>
+    <row r="481" ht="28" customHeight="1">
+      <c r="A481" s="16" t="inlineStr">
         <is>
           <t>MAE DU, 15 min, busy hour. Trial = CR01 10 gNB (or any cell where Section 3 was sent). Control = neighbour 32T not in the trial. Pre D−7, post D+1 and D+7. Source: FPD Counter Changes for MIMO TDD / Beam / AHR / iBeam / UL Boosting.</t>
         </is>
       </c>
-      <c r="B468" s="17" t="n"/>
-      <c r="C468" s="17" t="n"/>
-      <c r="D468" s="17" t="n"/>
-      <c r="E468" s="17" t="n"/>
-      <c r="F468" s="17" t="n"/>
-      <c r="G468" s="17" t="n"/>
-      <c r="H468" s="17" t="n"/>
-      <c r="I468" s="17" t="n"/>
-      <c r="J468" s="17" t="n"/>
-      <c r="K468" s="17" t="n"/>
-      <c r="L468" s="17" t="n"/>
-      <c r="M468" s="17" t="n"/>
-    </row>
-    <row r="469" ht="24" customHeight="1">
-      <c r="A469" s="134" t="inlineStr">
+      <c r="B481" s="17" t="n"/>
+      <c r="C481" s="17" t="n"/>
+      <c r="D481" s="17" t="n"/>
+      <c r="E481" s="17" t="n"/>
+      <c r="F481" s="17" t="n"/>
+      <c r="G481" s="17" t="n"/>
+      <c r="H481" s="17" t="n"/>
+      <c r="I481" s="17" t="n"/>
+      <c r="J481" s="17" t="n"/>
+      <c r="K481" s="17" t="n"/>
+      <c r="L481" s="17" t="n"/>
+      <c r="M481" s="17" t="n"/>
+    </row>
+    <row r="482" ht="24" customHeight="1">
+      <c r="A482" s="134" t="inlineStr">
         <is>
           <t>SN</t>
         </is>
       </c>
-      <c r="B469" s="134" t="inlineStr">
+      <c r="B482" s="134" t="inlineStr">
         <is>
           <t>Counter ID</t>
         </is>
       </c>
-      <c r="C469" s="134" t="inlineStr">
+      <c r="C482" s="134" t="inlineStr">
         <is>
           <t>Counter Name</t>
         </is>
       </c>
-      <c r="D469" s="134" t="inlineStr">
+      <c r="D482" s="134" t="inlineStr">
         <is>
           <t>Function</t>
         </is>
       </c>
-      <c r="E469" s="134" t="inlineStr">
+      <c r="E482" s="134" t="inlineStr">
         <is>
           <t>Use for Section 1 suggestions</t>
         </is>
       </c>
-      <c r="F469" s="134" t="inlineStr">
+      <c r="F482" s="134" t="inlineStr">
         <is>
           <t>KPI it feeds</t>
         </is>
       </c>
-      <c r="G469" s="134" t="inlineStr">
+      <c r="G482" s="134" t="inlineStr">
         <is>
           <t>Granularity</t>
         </is>
       </c>
-      <c r="H469" s="134" t="inlineStr">
+      <c r="H482" s="134" t="inlineStr">
         <is>
           <t>Pass / fail gate</t>
         </is>
       </c>
-      <c r="I469" s="134" t="inlineStr"/>
-      <c r="J469" s="134" t="inlineStr"/>
-      <c r="K469" s="134" t="inlineStr"/>
-      <c r="L469" s="134" t="inlineStr"/>
-      <c r="M469" s="134" t="inlineStr"/>
-    </row>
-    <row r="470" ht="42" customHeight="1">
-      <c r="A470" s="143" t="n">
+      <c r="I482" s="134" t="inlineStr"/>
+      <c r="J482" s="134" t="inlineStr"/>
+      <c r="K482" s="134" t="inlineStr"/>
+      <c r="L482" s="134" t="inlineStr"/>
+      <c r="M482" s="134" t="inlineStr"/>
+    </row>
+    <row r="483" ht="42" customHeight="1">
+      <c r="A483" s="143" t="n">
         <v>1</v>
       </c>
-      <c r="B470" s="144" t="inlineStr">
+      <c r="B483" s="144" t="inlineStr">
         <is>
           <t>N.ThpVol.DL / N.RLC.ThpTime.DL.Cell</t>
         </is>
       </c>
-      <c r="C470" s="144" t="inlineStr">
+      <c r="C483" s="144" t="inlineStr">
         <is>
           <t>User DL Average Throughput (DU)</t>
         </is>
       </c>
-      <c r="D470" s="145" t="inlineStr">
+      <c r="D483" s="145" t="inlineStr">
         <is>
           <t>North-star commercial KPI for every DL box (S15-01..16, 25).</t>
         </is>
       </c>
-      <c r="E470" s="145" t="inlineStr">
+      <c r="E483" s="145" t="inlineStr">
         <is>
           <t>Must not drop vs control. Target: lift vs pre-CR week.</t>
         </is>
       </c>
-      <c r="F470" s="145" t="inlineStr">
+      <c r="F483" s="145" t="inlineStr">
         <is>
           <t>User DL Average Throughput (DU)</t>
         </is>
       </c>
-      <c r="G470" s="145" t="inlineStr">
+      <c r="G483" s="145" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H470" s="145" t="inlineStr">
+      <c r="H483" s="145" t="inlineStr">
         <is>
           <t>Fail if trial &lt; control trend.</t>
         </is>
       </c>
-      <c r="I470" s="145" t="inlineStr"/>
-      <c r="J470" s="145" t="inlineStr"/>
-      <c r="K470" s="145" t="inlineStr"/>
-      <c r="L470" s="145" t="inlineStr"/>
-      <c r="M470" s="145" t="inlineStr"/>
-    </row>
-    <row r="471" ht="42" customHeight="1">
-      <c r="A471" s="146" t="n">
+      <c r="I483" s="145" t="inlineStr"/>
+      <c r="J483" s="145" t="inlineStr"/>
+      <c r="K483" s="145" t="inlineStr"/>
+      <c r="L483" s="145" t="inlineStr"/>
+      <c r="M483" s="145" t="inlineStr"/>
+    </row>
+    <row r="484" ht="42" customHeight="1">
+      <c r="A484" s="146" t="n">
         <v>2</v>
       </c>
-      <c r="B471" s="147" t="inlineStr">
+      <c r="B484" s="147" t="inlineStr">
         <is>
           <t>N.ThpVol.UL / N.RLC.ThpTime.UL.Cell</t>
         </is>
       </c>
-      <c r="C471" s="147" t="inlineStr">
+      <c r="C484" s="147" t="inlineStr">
         <is>
           <t>User UL Average Throughput (DU)</t>
         </is>
       </c>
-      <c r="D471" s="36" t="inlineStr">
+      <c r="D484" s="36" t="inlineStr">
         <is>
           <t>UL boxes S15-03 / 10 / 19 / 20 and SRS quality that feeds DL weights.</t>
         </is>
       </c>
-      <c r="E471" s="36" t="inlineStr">
+      <c r="E484" s="36" t="inlineStr">
         <is>
           <t>UL Boosting + PUSCH CE + UL rank.</t>
         </is>
       </c>
-      <c r="F471" s="36" t="inlineStr">
+      <c r="F484" s="36" t="inlineStr">
         <is>
           <t>User UL Average Throughput (DU)</t>
         </is>
       </c>
-      <c r="G471" s="36" t="inlineStr">
+      <c r="G484" s="36" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H471" s="36" t="inlineStr">
+      <c r="H484" s="36" t="inlineStr">
         <is>
           <t>Fail if UL regresses.</t>
         </is>
       </c>
-      <c r="I471" s="36" t="inlineStr"/>
-      <c r="J471" s="36" t="inlineStr"/>
-      <c r="K471" s="36" t="inlineStr"/>
-      <c r="L471" s="36" t="inlineStr"/>
-      <c r="M471" s="36" t="inlineStr"/>
-    </row>
-    <row r="472" ht="42" customHeight="1">
-      <c r="A472" s="143" t="n">
+      <c r="I484" s="36" t="inlineStr"/>
+      <c r="J484" s="36" t="inlineStr"/>
+      <c r="K484" s="36" t="inlineStr"/>
+      <c r="L484" s="36" t="inlineStr"/>
+      <c r="M484" s="36" t="inlineStr"/>
+    </row>
+    <row r="485" ht="42" customHeight="1">
+      <c r="A485" s="143" t="n">
         <v>3</v>
       </c>
-      <c r="B472" s="144" t="inlineStr">
+      <c r="B485" s="144" t="inlineStr">
         <is>
           <t>N.DL.SCH.*.ErrTB.Ibler / N.DL.SCH.*.TB</t>
         </is>
       </c>
-      <c r="C472" s="144" t="inlineStr">
+      <c r="C485" s="144" t="inlineStr">
         <is>
           <t>DL IBLER by MCS</t>
         </is>
       </c>
-      <c r="D472" s="145" t="inlineStr">
+      <c r="D485" s="145" t="inlineStr">
         <is>
           <t>iBeam precise/anti-intrf, tail-pkt MCS, hybrid IR (S15-16).</t>
         </is>
       </c>
-      <c r="E472" s="145" t="inlineStr">
+      <c r="E485" s="145" t="inlineStr">
         <is>
           <t>Gate for MU/iBeam.</t>
         </is>
       </c>
-      <c r="F472" s="145" t="inlineStr">
+      <c r="F485" s="145" t="inlineStr">
         <is>
           <t>DL IBLER %</t>
         </is>
       </c>
-      <c r="G472" s="145" t="inlineStr">
+      <c r="G485" s="145" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H472" s="145" t="inlineStr">
+      <c r="H485" s="145" t="inlineStr">
         <is>
           <t>Fail if IBLER jumps vs control.</t>
         </is>
       </c>
-      <c r="I472" s="145" t="inlineStr"/>
-      <c r="J472" s="145" t="inlineStr"/>
-      <c r="K472" s="145" t="inlineStr"/>
-      <c r="L472" s="145" t="inlineStr"/>
-      <c r="M472" s="145" t="inlineStr"/>
-    </row>
-    <row r="473" ht="42" customHeight="1">
-      <c r="A473" s="146" t="n">
+      <c r="I485" s="145" t="inlineStr"/>
+      <c r="J485" s="145" t="inlineStr"/>
+      <c r="K485" s="145" t="inlineStr"/>
+      <c r="L485" s="145" t="inlineStr"/>
+      <c r="M485" s="145" t="inlineStr"/>
+    </row>
+    <row r="486" ht="42" customHeight="1">
+      <c r="A486" s="146" t="n">
         <v>4</v>
       </c>
-      <c r="B473" s="147" t="inlineStr">
+      <c r="B486" s="147" t="inlineStr">
         <is>
           <t>N.UL.SCH.*.ErrTB.Ibler / .TB</t>
         </is>
       </c>
-      <c r="C473" s="147" t="inlineStr">
+      <c r="C486" s="147" t="inlineStr">
         <is>
           <t>UL IBLER</t>
         </is>
       </c>
-      <c r="D473" s="36" t="inlineStr">
+      <c r="D486" s="36" t="inlineStr">
         <is>
           <t>S15-03 rank/CE and S15-19 UL Boosting.</t>
         </is>
       </c>
-      <c r="E473" s="36" t="inlineStr">
+      <c r="E486" s="36" t="inlineStr">
         <is>
           <t>UL residual BLER.</t>
         </is>
       </c>
-      <c r="F473" s="36" t="inlineStr">
+      <c r="F486" s="36" t="inlineStr">
         <is>
           <t>UL IBLER %</t>
         </is>
       </c>
-      <c r="G473" s="36" t="inlineStr">
+      <c r="G486" s="36" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H473" s="36" t="inlineStr">
+      <c r="H486" s="36" t="inlineStr">
         <is>
           <t>Fail if UL IBLER jumps.</t>
         </is>
       </c>
-      <c r="I473" s="36" t="inlineStr"/>
-      <c r="J473" s="36" t="inlineStr"/>
-      <c r="K473" s="36" t="inlineStr"/>
-      <c r="L473" s="36" t="inlineStr"/>
-      <c r="M473" s="36" t="inlineStr"/>
-    </row>
-    <row r="474" ht="42" customHeight="1">
-      <c r="A474" s="143" t="n">
+      <c r="I486" s="36" t="inlineStr"/>
+      <c r="J486" s="36" t="inlineStr"/>
+      <c r="K486" s="36" t="inlineStr"/>
+      <c r="L486" s="36" t="inlineStr"/>
+      <c r="M486" s="36" t="inlineStr"/>
+    </row>
+    <row r="487" ht="42" customHeight="1">
+      <c r="A487" s="143" t="n">
         <v>5</v>
       </c>
-      <c r="B474" s="144" t="inlineStr">
+      <c r="B487" s="144" t="inlineStr">
         <is>
           <t>N.UL.SRS.PreSINR.Index* / N.SRS.NI.Avg</t>
         </is>
       </c>
-      <c r="C474" s="144" t="inlineStr">
+      <c r="C487" s="144" t="inlineStr">
         <is>
           <t>SRS quality / SRS NI</t>
         </is>
       </c>
-      <c r="D474" s="145" t="inlineStr">
+      <c r="D487" s="145" t="inlineStr">
         <is>
           <t>S15-02 weights, S15-14 joint PC, S15-16 tight MUX / blind IS.</t>
         </is>
       </c>
-      <c r="E474" s="145" t="inlineStr">
+      <c r="E487" s="145" t="inlineStr">
         <is>
           <t>SRS that drives DL BF.</t>
         </is>
       </c>
-      <c r="F474" s="145" t="inlineStr">
+      <c r="F487" s="145" t="inlineStr">
         <is>
           <t>SRS PreSINR / NI</t>
         </is>
       </c>
-      <c r="G474" s="145" t="inlineStr">
+      <c r="G487" s="145" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H474" s="145" t="inlineStr">
+      <c r="H487" s="145" t="inlineStr">
         <is>
           <t>Fail if NI jumps — do not add SRS_IC.</t>
         </is>
       </c>
-      <c r="I474" s="145" t="inlineStr"/>
-      <c r="J474" s="145" t="inlineStr"/>
-      <c r="K474" s="145" t="inlineStr"/>
-      <c r="L474" s="145" t="inlineStr"/>
-      <c r="M474" s="145" t="inlineStr"/>
-    </row>
-    <row r="475" ht="42" customHeight="1">
-      <c r="A475" s="146" t="n">
+      <c r="I487" s="145" t="inlineStr"/>
+      <c r="J487" s="145" t="inlineStr"/>
+      <c r="K487" s="145" t="inlineStr"/>
+      <c r="L487" s="145" t="inlineStr"/>
+      <c r="M487" s="145" t="inlineStr"/>
+    </row>
+    <row r="488" ht="42" customHeight="1">
+      <c r="A488" s="146" t="n">
         <v>6</v>
       </c>
-      <c r="B475" s="147" t="inlineStr">
+      <c r="B488" s="147" t="inlineStr">
         <is>
           <t>N.ChMeas.PDSCH.MCS.k / N.PDSCH.InitTbDl.Rank*</t>
         </is>
       </c>
-      <c r="C475" s="147" t="inlineStr">
+      <c r="C488" s="147" t="inlineStr">
         <is>
           <t>DL MCS / rank</t>
         </is>
       </c>
-      <c r="D475" s="36" t="inlineStr">
+      <c r="D488" s="36" t="inlineStr">
         <is>
           <t>S15-02 / 12 tracking / 16 iBeam.</t>
         </is>
       </c>
-      <c r="E475" s="36" t="inlineStr">
+      <c r="E488" s="36" t="inlineStr">
         <is>
           <t>BF gain = MCS upshift at same load.</t>
         </is>
       </c>
-      <c r="F475" s="36" t="inlineStr">
+      <c r="F488" s="36" t="inlineStr">
         <is>
           <t>MCS / rank mix</t>
         </is>
       </c>
-      <c r="G475" s="36" t="inlineStr">
+      <c r="G488" s="36" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H475" s="36" t="inlineStr">
+      <c r="H488" s="36" t="inlineStr">
         <is>
           <t>Informational with IBLER gate.</t>
         </is>
       </c>
-      <c r="I475" s="36" t="inlineStr"/>
-      <c r="J475" s="36" t="inlineStr"/>
-      <c r="K475" s="36" t="inlineStr"/>
-      <c r="L475" s="36" t="inlineStr"/>
-      <c r="M475" s="36" t="inlineStr"/>
-    </row>
-    <row r="476" ht="42" customHeight="1">
-      <c r="A476" s="143" t="n">
+      <c r="I488" s="36" t="inlineStr"/>
+      <c r="J488" s="36" t="inlineStr"/>
+      <c r="K488" s="36" t="inlineStr"/>
+      <c r="L488" s="36" t="inlineStr"/>
+      <c r="M488" s="36" t="inlineStr"/>
+    </row>
+    <row r="489" ht="42" customHeight="1">
+      <c r="A489" s="143" t="n">
         <v>7</v>
       </c>
-      <c r="B476" s="144" t="inlineStr">
+      <c r="B489" s="144" t="inlineStr">
         <is>
           <t>N.ChMeas.MIMO.DL.Pair.Layer.Avg / Pair.PRB</t>
         </is>
       </c>
-      <c r="C476" s="144" t="inlineStr">
+      <c r="C489" s="144" t="inlineStr">
         <is>
           <t>DL MU pairing</t>
         </is>
       </c>
-      <c r="D476" s="145" t="inlineStr">
+      <c r="D489" s="145" t="inlineStr">
         <is>
           <t>S15-07 already ON; S15-16 precise/anti-intrf; S15-09 later.</t>
         </is>
       </c>
-      <c r="E476" s="145" t="inlineStr">
+      <c r="E489" s="145" t="inlineStr">
         <is>
           <t>Pairing quality not raw count.</t>
         </is>
       </c>
-      <c r="F476" s="145" t="inlineStr">
+      <c r="F489" s="145" t="inlineStr">
         <is>
           <t>MU layers / PRB</t>
         </is>
       </c>
-      <c r="G476" s="145" t="inlineStr">
+      <c r="G489" s="145" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H476" s="145" t="inlineStr">
+      <c r="H489" s="145" t="inlineStr">
         <is>
           <t>Pairing up + IBLER up = rollback MU extras.</t>
         </is>
       </c>
-      <c r="I476" s="145" t="inlineStr"/>
-      <c r="J476" s="145" t="inlineStr"/>
-      <c r="K476" s="145" t="inlineStr"/>
-      <c r="L476" s="145" t="inlineStr"/>
-      <c r="M476" s="145" t="inlineStr"/>
-    </row>
-    <row r="477" ht="42" customHeight="1">
-      <c r="A477" s="146" t="n">
+      <c r="I489" s="145" t="inlineStr"/>
+      <c r="J489" s="145" t="inlineStr"/>
+      <c r="K489" s="145" t="inlineStr"/>
+      <c r="L489" s="145" t="inlineStr"/>
+      <c r="M489" s="145" t="inlineStr"/>
+    </row>
+    <row r="490" ht="42" customHeight="1">
+      <c r="A490" s="146" t="n">
         <v>8</v>
       </c>
-      <c r="B477" s="147" t="inlineStr">
+      <c r="B490" s="147" t="inlineStr">
         <is>
           <t>N.ChMeas.MIMO.UL.Pair.Layer / Pair.PRB</t>
         </is>
       </c>
-      <c r="C477" s="147" t="inlineStr">
+      <c r="C490" s="147" t="inlineStr">
         <is>
           <t>UL MU pairing</t>
         </is>
       </c>
-      <c r="D477" s="36" t="inlineStr">
+      <c r="D490" s="36" t="inlineStr">
         <is>
           <t>S15-19 CR01 children.</t>
         </is>
       </c>
-      <c r="E477" s="36" t="inlineStr">
+      <c r="E490" s="36" t="inlineStr">
         <is>
           <t>UL Boosting pairing.</t>
         </is>
       </c>
-      <c r="F477" s="36" t="inlineStr">
+      <c r="F490" s="36" t="inlineStr">
         <is>
           <t>UL MU layers / PRB</t>
         </is>
       </c>
-      <c r="G477" s="36" t="inlineStr">
+      <c r="G490" s="36" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H477" s="36" t="inlineStr">
+      <c r="H490" s="36" t="inlineStr">
         <is>
           <t>With UL IBLER.</t>
         </is>
       </c>
-      <c r="I477" s="36" t="inlineStr"/>
-      <c r="J477" s="36" t="inlineStr"/>
-      <c r="K477" s="36" t="inlineStr"/>
-      <c r="L477" s="36" t="inlineStr"/>
-      <c r="M477" s="36" t="inlineStr"/>
-    </row>
-    <row r="478" ht="42" customHeight="1">
-      <c r="A478" s="143" t="n">
+      <c r="I490" s="36" t="inlineStr"/>
+      <c r="J490" s="36" t="inlineStr"/>
+      <c r="K490" s="36" t="inlineStr"/>
+      <c r="L490" s="36" t="inlineStr"/>
+      <c r="M490" s="36" t="inlineStr"/>
+    </row>
+    <row r="491" ht="42" customHeight="1">
+      <c r="A491" s="143" t="n">
         <v>9</v>
       </c>
-      <c r="B478" s="144" t="inlineStr">
+      <c r="B491" s="144" t="inlineStr">
         <is>
           <t>N.CCE.DL.AllocReq.Num / N.CCE.DL.AggLvl* / N.CCE.Used.Avg</t>
         </is>
       </c>
-      <c r="C478" s="144" t="inlineStr">
+      <c r="C491" s="144" t="inlineStr">
         <is>
           <t>PDCCH CCE / agg-level</t>
         </is>
       </c>
-      <c r="D478" s="145" t="inlineStr">
+      <c r="D491" s="145" t="inlineStr">
         <is>
           <t>S15-16 PDCCH_AGG_LVL_COMPR.</t>
         </is>
       </c>
-      <c r="E478" s="145" t="inlineStr">
+      <c r="E491" s="145" t="inlineStr">
         <is>
           <t>Blocking proxy.</t>
         </is>
       </c>
-      <c r="F478" s="145" t="inlineStr">
+      <c r="F491" s="145" t="inlineStr">
         <is>
           <t>PDCCH CCE utilisation</t>
         </is>
       </c>
-      <c r="G478" s="145" t="inlineStr">
+      <c r="G491" s="145" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H478" s="145" t="inlineStr">
+      <c r="H491" s="145" t="inlineStr">
         <is>
           <t>Fail if blocking rises.</t>
         </is>
       </c>
-      <c r="I478" s="145" t="inlineStr"/>
-      <c r="J478" s="145" t="inlineStr"/>
-      <c r="K478" s="145" t="inlineStr"/>
-      <c r="L478" s="145" t="inlineStr"/>
-      <c r="M478" s="145" t="inlineStr"/>
-    </row>
-    <row r="479" ht="42" customHeight="1">
-      <c r="A479" s="146" t="n">
+      <c r="I491" s="145" t="inlineStr"/>
+      <c r="J491" s="145" t="inlineStr"/>
+      <c r="K491" s="145" t="inlineStr"/>
+      <c r="L491" s="145" t="inlineStr"/>
+      <c r="M491" s="145" t="inlineStr"/>
+    </row>
+    <row r="492" ht="42" customHeight="1">
+      <c r="A492" s="146" t="n">
         <v>10</v>
       </c>
-      <c r="B479" s="147" t="inlineStr">
+      <c r="B492" s="147" t="inlineStr">
         <is>
           <t>N.User.OptimalSSBBeam.Avg / N.MAC.ThpVol.DL.OptimalSSB</t>
         </is>
       </c>
-      <c r="C479" s="147" t="inlineStr">
+      <c r="C492" s="147" t="inlineStr">
         <is>
           <t>Optimal SSB users / volume</t>
         </is>
       </c>
-      <c r="D479" s="36" t="inlineStr">
+      <c r="D492" s="36" t="inlineStr">
         <is>
           <t>S15-12 SSB adapt + tracking.</t>
         </is>
       </c>
-      <c r="E479" s="36" t="inlineStr">
+      <c r="E492" s="36" t="inlineStr">
         <is>
           <t>Broadcast-beam follow.</t>
         </is>
       </c>
-      <c r="F479" s="36" t="inlineStr">
+      <c r="F492" s="36" t="inlineStr">
         <is>
           <t>SSB coverage</t>
         </is>
       </c>
-      <c r="G479" s="36" t="inlineStr">
+      <c r="G492" s="36" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H479" s="36" t="inlineStr">
+      <c r="H492" s="36" t="inlineStr">
         <is>
           <t>Drop/HO rise = rollback SSB bits.</t>
         </is>
       </c>
-      <c r="I479" s="36" t="inlineStr"/>
-      <c r="J479" s="36" t="inlineStr"/>
-      <c r="K479" s="36" t="inlineStr"/>
-      <c r="L479" s="36" t="inlineStr"/>
-      <c r="M479" s="36" t="inlineStr"/>
-    </row>
-    <row r="480" ht="42" customHeight="1">
-      <c r="A480" s="143" t="n">
+      <c r="I492" s="36" t="inlineStr"/>
+      <c r="J492" s="36" t="inlineStr"/>
+      <c r="K492" s="36" t="inlineStr"/>
+      <c r="L492" s="36" t="inlineStr"/>
+      <c r="M492" s="36" t="inlineStr"/>
+    </row>
+    <row r="493" ht="42" customHeight="1">
+      <c r="A493" s="143" t="n">
         <v>11</v>
       </c>
-      <c r="B480" s="144" t="inlineStr">
+      <c r="B493" s="144" t="inlineStr">
         <is>
           <t>N.ChMeas.CQI.SingleCW.k</t>
         </is>
       </c>
-      <c r="C480" s="144" t="inlineStr">
+      <c r="C493" s="144" t="inlineStr">
         <is>
           <t>Wideband CQI</t>
         </is>
       </c>
-      <c r="D480" s="145" t="inlineStr">
+      <c r="D493" s="145" t="inlineStr">
         <is>
           <t>S15-13 AHR Phase1 (already ON).</t>
         </is>
       </c>
-      <c r="E480" s="145" t="inlineStr">
+      <c r="E493" s="145" t="inlineStr">
         <is>
           <t>CSI quality baseline.</t>
         </is>
       </c>
-      <c r="F480" s="145" t="inlineStr">
+      <c r="F493" s="145" t="inlineStr">
         <is>
           <t>Average CQI</t>
         </is>
       </c>
-      <c r="G480" s="145" t="inlineStr">
+      <c r="G493" s="145" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H480" s="145" t="inlineStr">
+      <c r="H493" s="145" t="inlineStr">
         <is>
           <t>Should already be commercial-like.</t>
         </is>
       </c>
-      <c r="I480" s="145" t="inlineStr"/>
-      <c r="J480" s="145" t="inlineStr"/>
-      <c r="K480" s="145" t="inlineStr"/>
-      <c r="L480" s="145" t="inlineStr"/>
-      <c r="M480" s="145" t="inlineStr"/>
-    </row>
-    <row r="481" ht="42" customHeight="1">
-      <c r="A481" s="146" t="n">
+      <c r="I493" s="145" t="inlineStr"/>
+      <c r="J493" s="145" t="inlineStr"/>
+      <c r="K493" s="145" t="inlineStr"/>
+      <c r="L493" s="145" t="inlineStr"/>
+      <c r="M493" s="145" t="inlineStr"/>
+    </row>
+    <row r="494" ht="42" customHeight="1">
+      <c r="A494" s="146" t="n">
         <v>12</v>
       </c>
-      <c r="B481" s="147" t="inlineStr">
+      <c r="B494" s="147" t="inlineStr">
         <is>
           <t>N.ChMeas.MIMO.DL.Transmission.Layer.Max</t>
         </is>
       </c>
-      <c r="C481" s="147" t="inlineStr">
+      <c r="C494" s="147" t="inlineStr">
         <is>
           <t>Max DL layers on a PRB</t>
         </is>
       </c>
-      <c r="D481" s="36" t="inlineStr">
+      <c r="D494" s="36" t="inlineStr">
         <is>
           <t>S15-05 SU quota (LAYER_16 live). S15-09 spends it later.</t>
         </is>
       </c>
-      <c r="E481" s="36" t="inlineStr">
+      <c r="E494" s="36" t="inlineStr">
         <is>
           <t>Layer consumption.</t>
         </is>
       </c>
-      <c r="F481" s="36" t="inlineStr">
+      <c r="F494" s="36" t="inlineStr">
         <is>
           <t>Max DL layers</t>
         </is>
       </c>
-      <c r="G481" s="36" t="inlineStr">
+      <c r="G494" s="36" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H481" s="36" t="inlineStr">
+      <c r="H494" s="36" t="inlineStr">
         <is>
           <t>Do not drop after any MOD.</t>
         </is>
       </c>
-      <c r="I481" s="36" t="inlineStr"/>
-      <c r="J481" s="36" t="inlineStr"/>
-      <c r="K481" s="36" t="inlineStr"/>
-      <c r="L481" s="36" t="inlineStr"/>
-      <c r="M481" s="36" t="inlineStr"/>
-    </row>
-    <row r="482" ht="42" customHeight="1">
-      <c r="A482" s="143" t="n">
+      <c r="I494" s="36" t="inlineStr"/>
+      <c r="J494" s="36" t="inlineStr"/>
+      <c r="K494" s="36" t="inlineStr"/>
+      <c r="L494" s="36" t="inlineStr"/>
+      <c r="M494" s="36" t="inlineStr"/>
+    </row>
+    <row r="495" ht="42" customHeight="1">
+      <c r="A495" s="143" t="n">
         <v>13</v>
       </c>
-      <c r="B482" s="144" t="inlineStr">
+      <c r="B495" s="144" t="inlineStr">
         <is>
           <t>N.UECntx.AbnormRel / N.RRC.ReEst.Att</t>
         </is>
       </c>
-      <c r="C482" s="144" t="inlineStr">
+      <c r="C495" s="144" t="inlineStr">
         <is>
           <t>Drop / re-establish</t>
         </is>
       </c>
-      <c r="D482" s="145" t="inlineStr">
+      <c r="D495" s="145" t="inlineStr">
         <is>
           <t>Safety for S15-12 SSB + S15-16 iBeam in one window.</t>
         </is>
       </c>
-      <c r="E482" s="145" t="inlineStr">
+      <c r="E495" s="145" t="inlineStr">
         <is>
           <t>Must not rise.</t>
         </is>
       </c>
-      <c r="F482" s="145" t="inlineStr">
+      <c r="F495" s="145" t="inlineStr">
         <is>
           <t>Drop / re-est</t>
         </is>
       </c>
-      <c r="G482" s="145" t="inlineStr">
+      <c r="G495" s="145" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H482" s="145" t="inlineStr">
+      <c r="H495" s="145" t="inlineStr">
         <is>
           <t>Any rise vs control → rollback that gNB.</t>
         </is>
       </c>
-      <c r="I482" s="145" t="inlineStr"/>
-      <c r="J482" s="145" t="inlineStr"/>
-      <c r="K482" s="145" t="inlineStr"/>
-      <c r="L482" s="145" t="inlineStr"/>
-      <c r="M482" s="145" t="inlineStr"/>
-    </row>
-    <row r="483" ht="42" customHeight="1">
-      <c r="A483" s="146" t="n">
+      <c r="I495" s="145" t="inlineStr"/>
+      <c r="J495" s="145" t="inlineStr"/>
+      <c r="K495" s="145" t="inlineStr"/>
+      <c r="L495" s="145" t="inlineStr"/>
+      <c r="M495" s="145" t="inlineStr"/>
+    </row>
+    <row r="496" ht="42" customHeight="1">
+      <c r="A496" s="146" t="n">
         <v>14</v>
       </c>
-      <c r="B483" s="147" t="inlineStr">
+      <c r="B496" s="147" t="inlineStr">
         <is>
           <t>N.PRB.DL.Used.Avg / N.PRB.UL.Used.Avg</t>
         </is>
       </c>
-      <c r="C483" s="147" t="inlineStr">
+      <c r="C496" s="147" t="inlineStr">
         <is>
           <t>PRB usage (load)</t>
         </is>
       </c>
-      <c r="D483" s="36" t="inlineStr">
+      <c r="D496" s="36" t="inlineStr">
         <is>
           <t>Normalise every tput/MCS comparison.</t>
         </is>
       </c>
-      <c r="E483" s="36" t="inlineStr">
+      <c r="E496" s="36" t="inlineStr">
         <is>
           <t>Same BH, similar load.</t>
         </is>
       </c>
-      <c r="F483" s="36" t="inlineStr">
+      <c r="F496" s="36" t="inlineStr">
         <is>
           <t>PRB %</t>
         </is>
       </c>
-      <c r="G483" s="36" t="inlineStr">
+      <c r="G496" s="36" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H483" s="36" t="inlineStr">
+      <c r="H496" s="36" t="inlineStr">
         <is>
           <t>Do not compare empty vs loaded cells.</t>
         </is>
       </c>
-      <c r="I483" s="36" t="inlineStr"/>
-      <c r="J483" s="36" t="inlineStr"/>
-      <c r="K483" s="36" t="inlineStr"/>
-      <c r="L483" s="36" t="inlineStr"/>
-      <c r="M483" s="36" t="inlineStr"/>
-    </row>
-    <row r="484" ht="42" customHeight="1">
-      <c r="A484" s="143" t="n">
+      <c r="I496" s="36" t="inlineStr"/>
+      <c r="J496" s="36" t="inlineStr"/>
+      <c r="K496" s="36" t="inlineStr"/>
+      <c r="L496" s="36" t="inlineStr"/>
+      <c r="M496" s="36" t="inlineStr"/>
+    </row>
+    <row r="497" ht="42" customHeight="1">
+      <c r="A497" s="143" t="n">
         <v>15</v>
       </c>
-      <c r="B484" s="144" t="inlineStr">
+      <c r="B497" s="144" t="inlineStr">
         <is>
           <t>N.QoS.DL.PktDelayAirInterface.* / N.Traffic.DL.RlcFirstPktDelay.Time</t>
         </is>
       </c>
-      <c r="C484" s="144" t="inlineStr">
+      <c r="C497" s="144" t="inlineStr">
         <is>
           <t>DL latency / first-packet delay</t>
         </is>
       </c>
-      <c r="D484" s="145" t="inlineStr">
+      <c r="D497" s="145" t="inlineStr">
         <is>
           <t>S15-16 RLC merge + res-based adapt sch.</t>
         </is>
       </c>
-      <c r="E484" s="145" t="inlineStr">
+      <c r="E497" s="145" t="inlineStr">
         <is>
           <t>Tail experience.</t>
         </is>
       </c>
-      <c r="F484" s="145" t="inlineStr">
+      <c r="F497" s="145" t="inlineStr">
         <is>
           <t>Delay ms</t>
         </is>
       </c>
-      <c r="G484" s="145" t="inlineStr">
+      <c r="G497" s="145" t="inlineStr">
         <is>
           <t>15 min / cell</t>
         </is>
       </c>
-      <c r="H484" s="145" t="inlineStr">
+      <c r="H497" s="145" t="inlineStr">
         <is>
           <t>Should not rise.</t>
         </is>
       </c>
-      <c r="I484" s="145" t="inlineStr"/>
-      <c r="J484" s="145" t="inlineStr"/>
-      <c r="K484" s="145" t="inlineStr"/>
-      <c r="L484" s="145" t="inlineStr"/>
-      <c r="M484" s="145" t="inlineStr"/>
-    </row>
-    <row r="485" ht="8" customHeight="1"/>
-    <row r="486" ht="20" customHeight="1">
-      <c r="A486" s="30" t="inlineStr">
+      <c r="I497" s="145" t="inlineStr"/>
+      <c r="J497" s="145" t="inlineStr"/>
+      <c r="K497" s="145" t="inlineStr"/>
+      <c r="L497" s="145" t="inlineStr"/>
+      <c r="M497" s="145" t="inlineStr"/>
+    </row>
+    <row r="498" ht="8" customHeight="1"/>
+    <row r="499" ht="20" customHeight="1">
+      <c r="A499" s="30" t="inlineStr">
         <is>
           <t>MAE KPI (derived)</t>
         </is>
       </c>
-      <c r="B486" s="6" t="n"/>
-      <c r="C486" s="6" t="n"/>
-      <c r="D486" s="6" t="n"/>
-      <c r="E486" s="6" t="n"/>
-      <c r="F486" s="6" t="n"/>
-      <c r="G486" s="6" t="n"/>
-      <c r="H486" s="6" t="n"/>
-      <c r="I486" s="6" t="n"/>
-      <c r="J486" s="6" t="n"/>
-      <c r="K486" s="6" t="n"/>
-      <c r="L486" s="6" t="n"/>
-      <c r="M486" s="6" t="n"/>
-    </row>
-    <row r="487" ht="22" customHeight="1">
-      <c r="A487" s="7" t="inlineStr">
+      <c r="B499" s="6" t="n"/>
+      <c r="C499" s="6" t="n"/>
+      <c r="D499" s="6" t="n"/>
+      <c r="E499" s="6" t="n"/>
+      <c r="F499" s="6" t="n"/>
+      <c r="G499" s="6" t="n"/>
+      <c r="H499" s="6" t="n"/>
+      <c r="I499" s="6" t="n"/>
+      <c r="J499" s="6" t="n"/>
+      <c r="K499" s="6" t="n"/>
+      <c r="L499" s="6" t="n"/>
+      <c r="M499" s="6" t="n"/>
+    </row>
+    <row r="500" ht="22" customHeight="1">
+      <c r="A500" s="7" t="inlineStr">
         <is>
           <t>SN</t>
         </is>
       </c>
-      <c r="B487" s="7" t="inlineStr">
+      <c r="B500" s="7" t="inlineStr">
         <is>
           <t>KPI</t>
         </is>
       </c>
-      <c r="C487" s="7" t="inlineStr">
+      <c r="C500" s="7" t="inlineStr">
         <is>
           <t>Formula (from document)</t>
         </is>
       </c>
-      <c r="D487" s="7" t="inlineStr">
+      <c r="D500" s="7" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="E487" s="7" t="inlineStr">
+      <c r="E500" s="7" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="F487" s="7" t="inlineStr"/>
-      <c r="G487" s="7" t="inlineStr"/>
-      <c r="H487" s="7" t="inlineStr"/>
-      <c r="I487" s="7" t="inlineStr"/>
-      <c r="J487" s="7" t="inlineStr"/>
-    </row>
-    <row r="488" ht="36" customHeight="1">
-      <c r="A488" s="24" t="n">
+      <c r="F500" s="7" t="inlineStr"/>
+      <c r="G500" s="7" t="inlineStr"/>
+      <c r="H500" s="7" t="inlineStr"/>
+      <c r="I500" s="7" t="inlineStr"/>
+      <c r="J500" s="7" t="inlineStr"/>
+    </row>
+    <row r="501" ht="36" customHeight="1">
+      <c r="A501" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="B488" s="25" t="inlineStr">
+      <c r="B501" s="25" t="inlineStr">
         <is>
           <t>User DL Average Throughput (DU)</t>
         </is>
       </c>
-      <c r="C488" s="12" t="inlineStr">
+      <c r="C501" s="12" t="inlineStr">
         <is>
           <t>N.ThpVol.DL / N.RLC.ThpTime.DL.Cell (MAE)</t>
         </is>
       </c>
-      <c r="D488" s="12" t="inlineStr">
+      <c r="D501" s="12" t="inlineStr">
         <is>
           <t>Mbit/s</t>
         </is>
       </c>
-      <c r="E488" s="12" t="inlineStr">
+      <c r="E501" s="12" t="inlineStr">
         <is>
           <t>Pass: no drop vs control. Target: lift vs D−7.</t>
         </is>
       </c>
-      <c r="F488" s="10" t="n"/>
-      <c r="G488" s="10" t="n"/>
-      <c r="H488" s="10" t="n"/>
-      <c r="I488" s="10" t="n"/>
-      <c r="J488" s="11" t="n"/>
-      <c r="K488" s="151" t="n"/>
-      <c r="L488" s="151" t="n"/>
-      <c r="M488" s="151" t="n"/>
-    </row>
-    <row r="489" ht="36" customHeight="1">
-      <c r="A489" s="26" t="n">
+      <c r="F501" s="10" t="n"/>
+      <c r="G501" s="10" t="n"/>
+      <c r="H501" s="10" t="n"/>
+      <c r="I501" s="10" t="n"/>
+      <c r="J501" s="11" t="n"/>
+      <c r="K501" s="151" t="n"/>
+      <c r="L501" s="151" t="n"/>
+      <c r="M501" s="151" t="n"/>
+    </row>
+    <row r="502" ht="36" customHeight="1">
+      <c r="A502" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="B489" s="27" t="inlineStr">
+      <c r="B502" s="27" t="inlineStr">
         <is>
           <t>User UL Average Throughput (DU)</t>
         </is>
       </c>
-      <c r="C489" s="9" t="inlineStr">
+      <c r="C502" s="9" t="inlineStr">
         <is>
           <t>N.ThpVol.UL / N.RLC.ThpTime.UL.Cell (MAE)</t>
         </is>
       </c>
-      <c r="D489" s="9" t="inlineStr">
+      <c r="D502" s="9" t="inlineStr">
         <is>
           <t>Mbit/s</t>
         </is>
       </c>
-      <c r="E489" s="9" t="inlineStr">
+      <c r="E502" s="9" t="inlineStr">
         <is>
           <t>Pass: no UL regression after Boosting/CE/rank.</t>
         </is>
       </c>
-      <c r="F489" s="10" t="n"/>
-      <c r="G489" s="10" t="n"/>
-      <c r="H489" s="10" t="n"/>
-      <c r="I489" s="10" t="n"/>
-      <c r="J489" s="11" t="n"/>
-      <c r="K489" s="152" t="n"/>
-      <c r="L489" s="152" t="n"/>
-      <c r="M489" s="152" t="n"/>
-    </row>
-    <row r="490" ht="36" customHeight="1">
-      <c r="A490" s="24" t="n">
+      <c r="F502" s="10" t="n"/>
+      <c r="G502" s="10" t="n"/>
+      <c r="H502" s="10" t="n"/>
+      <c r="I502" s="10" t="n"/>
+      <c r="J502" s="11" t="n"/>
+      <c r="K502" s="152" t="n"/>
+      <c r="L502" s="152" t="n"/>
+      <c r="M502" s="152" t="n"/>
+    </row>
+    <row r="503" ht="36" customHeight="1">
+      <c r="A503" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="B490" s="25" t="inlineStr">
+      <c r="B503" s="25" t="inlineStr">
         <is>
           <t>DL IBLER</t>
         </is>
       </c>
-      <c r="C490" s="12" t="inlineStr">
+      <c r="C503" s="12" t="inlineStr">
         <is>
           <t>Σ N.DL.SCH.*.ErrTB.Ibler / Σ N.DL.SCH.*.TB</t>
         </is>
       </c>
-      <c r="D490" s="12" t="inlineStr">
+      <c r="D503" s="12" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E490" s="12" t="inlineStr">
+      <c r="E503" s="12" t="inlineStr">
         <is>
           <t>Pass: within planned band vs control.</t>
         </is>
       </c>
-      <c r="F490" s="10" t="n"/>
-      <c r="G490" s="10" t="n"/>
-      <c r="H490" s="10" t="n"/>
-      <c r="I490" s="10" t="n"/>
-      <c r="J490" s="11" t="n"/>
-      <c r="K490" s="151" t="n"/>
-      <c r="L490" s="151" t="n"/>
-      <c r="M490" s="151" t="n"/>
-    </row>
-    <row r="491" ht="36" customHeight="1">
-      <c r="A491" s="26" t="n">
+      <c r="F503" s="10" t="n"/>
+      <c r="G503" s="10" t="n"/>
+      <c r="H503" s="10" t="n"/>
+      <c r="I503" s="10" t="n"/>
+      <c r="J503" s="11" t="n"/>
+      <c r="K503" s="151" t="n"/>
+      <c r="L503" s="151" t="n"/>
+      <c r="M503" s="151" t="n"/>
+    </row>
+    <row r="504" ht="36" customHeight="1">
+      <c r="A504" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="B491" s="27" t="inlineStr">
+      <c r="B504" s="27" t="inlineStr">
         <is>
           <t>UL IBLER</t>
         </is>
       </c>
-      <c r="C491" s="9" t="inlineStr">
+      <c r="C504" s="9" t="inlineStr">
         <is>
           <t>Σ N.UL.SCH.*.ErrTB.Ibler / Σ TB</t>
         </is>
       </c>
-      <c r="D491" s="9" t="inlineStr">
+      <c r="D504" s="9" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E491" s="9" t="inlineStr">
+      <c r="E504" s="9" t="inlineStr">
         <is>
           <t>Pass: no jump after UL_LOW_NOISE / rank fast decrease.</t>
         </is>
       </c>
-      <c r="F491" s="10" t="n"/>
-      <c r="G491" s="10" t="n"/>
-      <c r="H491" s="10" t="n"/>
-      <c r="I491" s="10" t="n"/>
-      <c r="J491" s="11" t="n"/>
-      <c r="K491" s="152" t="n"/>
-      <c r="L491" s="152" t="n"/>
-      <c r="M491" s="152" t="n"/>
-    </row>
-    <row r="492" ht="36" customHeight="1">
-      <c r="A492" s="24" t="n">
+      <c r="F504" s="10" t="n"/>
+      <c r="G504" s="10" t="n"/>
+      <c r="H504" s="10" t="n"/>
+      <c r="I504" s="10" t="n"/>
+      <c r="J504" s="11" t="n"/>
+      <c r="K504" s="152" t="n"/>
+      <c r="L504" s="152" t="n"/>
+      <c r="M504" s="152" t="n"/>
+    </row>
+    <row r="505" ht="36" customHeight="1">
+      <c r="A505" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B492" s="25" t="inlineStr">
+      <c r="B505" s="25" t="inlineStr">
         <is>
           <t>PDCCH CCE utilisation</t>
         </is>
       </c>
-      <c r="C492" s="12" t="inlineStr">
+      <c r="C505" s="12" t="inlineStr">
         <is>
           <t>N.CCE.Used.Avg / N.CCE.Avail.*</t>
         </is>
       </c>
-      <c r="D492" s="12" t="inlineStr">
+      <c r="D505" s="12" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E492" s="12" t="inlineStr">
+      <c r="E505" s="12" t="inlineStr">
         <is>
           <t>Pass: used CCE falls or holds after agg-compress.</t>
         </is>
       </c>
-      <c r="F492" s="10" t="n"/>
-      <c r="G492" s="10" t="n"/>
-      <c r="H492" s="10" t="n"/>
-      <c r="I492" s="10" t="n"/>
-      <c r="J492" s="11" t="n"/>
-      <c r="K492" s="151" t="n"/>
-      <c r="L492" s="151" t="n"/>
-      <c r="M492" s="151" t="n"/>
-    </row>
-    <row r="493" ht="36" customHeight="1">
-      <c r="A493" s="26" t="n">
+      <c r="F505" s="10" t="n"/>
+      <c r="G505" s="10" t="n"/>
+      <c r="H505" s="10" t="n"/>
+      <c r="I505" s="10" t="n"/>
+      <c r="J505" s="11" t="n"/>
+      <c r="K505" s="151" t="n"/>
+      <c r="L505" s="151" t="n"/>
+      <c r="M505" s="151" t="n"/>
+    </row>
+    <row r="506" ht="36" customHeight="1">
+      <c r="A506" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="B493" s="27" t="inlineStr">
+      <c r="B506" s="27" t="inlineStr">
         <is>
           <t>SSB optimal-beam users</t>
         </is>
       </c>
-      <c r="C493" s="9" t="inlineStr">
+      <c r="C506" s="9" t="inlineStr">
         <is>
           <t>N.User.OptimalSSBBeam.Avg</t>
         </is>
       </c>
-      <c r="D493" s="9" t="inlineStr">
+      <c r="D506" s="9" t="inlineStr">
         <is>
           <t>users</t>
         </is>
       </c>
-      <c r="E493" s="9" t="inlineStr">
+      <c r="E506" s="9" t="inlineStr">
         <is>
           <t>Should rise after SSB adapt; watch drop.</t>
         </is>
       </c>
-      <c r="F493" s="10" t="n"/>
-      <c r="G493" s="10" t="n"/>
-      <c r="H493" s="10" t="n"/>
-      <c r="I493" s="10" t="n"/>
-      <c r="J493" s="11" t="n"/>
-      <c r="K493" s="152" t="n"/>
-      <c r="L493" s="152" t="n"/>
-      <c r="M493" s="152" t="n"/>
+      <c r="F506" s="10" t="n"/>
+      <c r="G506" s="10" t="n"/>
+      <c r="H506" s="10" t="n"/>
+      <c r="I506" s="10" t="n"/>
+      <c r="J506" s="11" t="n"/>
+      <c r="K506" s="152" t="n"/>
+      <c r="L506" s="152" t="n"/>
+      <c r="M506" s="152" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="869">
+  <mergeCells count="881">
     <mergeCell ref="I257:J257"/>
     <mergeCell ref="K321:M321"/>
     <mergeCell ref="B209:F209"/>
@@ -27448,6 +27843,7 @@
     <mergeCell ref="B238:F238"/>
     <mergeCell ref="I106:J106"/>
     <mergeCell ref="I302:J302"/>
+    <mergeCell ref="F469:M469"/>
     <mergeCell ref="B303:F303"/>
     <mergeCell ref="K145:M145"/>
     <mergeCell ref="K316:M316"/>
@@ -27460,6 +27856,7 @@
     <mergeCell ref="K147:M147"/>
     <mergeCell ref="A260:M260"/>
     <mergeCell ref="A60:M60"/>
+    <mergeCell ref="F470:M470"/>
     <mergeCell ref="B313:M313"/>
     <mergeCell ref="C11:J11"/>
     <mergeCell ref="A196:J196"/>
@@ -27592,7 +27989,6 @@
     <mergeCell ref="B325:F325"/>
     <mergeCell ref="I364:J364"/>
     <mergeCell ref="L352:M352"/>
-    <mergeCell ref="A468:M468"/>
     <mergeCell ref="I65:J65"/>
     <mergeCell ref="K129:M129"/>
     <mergeCell ref="I192:J192"/>
@@ -27609,8 +28005,8 @@
     <mergeCell ref="I286:J286"/>
     <mergeCell ref="K350:M350"/>
     <mergeCell ref="B385:F385"/>
-    <mergeCell ref="E492:J492"/>
     <mergeCell ref="B86:F86"/>
+    <mergeCell ref="E502:J502"/>
     <mergeCell ref="B151:F151"/>
     <mergeCell ref="K287:M287"/>
     <mergeCell ref="L71:M71"/>
@@ -27652,7 +28048,6 @@
     <mergeCell ref="K282:M282"/>
     <mergeCell ref="A91:J91"/>
     <mergeCell ref="A72:M72"/>
-    <mergeCell ref="E490:J490"/>
     <mergeCell ref="I225:J225"/>
     <mergeCell ref="B180:F180"/>
     <mergeCell ref="A155:J155"/>
@@ -27673,7 +28068,6 @@
     <mergeCell ref="B172:F172"/>
     <mergeCell ref="B270:F270"/>
     <mergeCell ref="K124:M124"/>
-    <mergeCell ref="E493:J493"/>
     <mergeCell ref="B257:F257"/>
     <mergeCell ref="K360:M360"/>
     <mergeCell ref="B288:F288"/>
@@ -27716,7 +28110,6 @@
     <mergeCell ref="I162:J162"/>
     <mergeCell ref="K283:M283"/>
     <mergeCell ref="A241:J241"/>
-    <mergeCell ref="A467:M467"/>
     <mergeCell ref="K274:M274"/>
     <mergeCell ref="A228:J228"/>
     <mergeCell ref="I373:J373"/>
@@ -27764,6 +28157,7 @@
     <mergeCell ref="K269:M269"/>
     <mergeCell ref="K296:M296"/>
     <mergeCell ref="A353:M353"/>
+    <mergeCell ref="A480:M480"/>
     <mergeCell ref="B137:M137"/>
     <mergeCell ref="I150:J150"/>
     <mergeCell ref="I321:J321"/>
@@ -27783,6 +28177,7 @@
     <mergeCell ref="B255:F255"/>
     <mergeCell ref="B364:F364"/>
     <mergeCell ref="K218:M218"/>
+    <mergeCell ref="F475:M475"/>
     <mergeCell ref="B65:F65"/>
     <mergeCell ref="C17:J17"/>
     <mergeCell ref="K24:M24"/>
@@ -27794,6 +28189,7 @@
     <mergeCell ref="B284:F284"/>
     <mergeCell ref="B222:F222"/>
     <mergeCell ref="K309:M309"/>
+    <mergeCell ref="F468:M468"/>
     <mergeCell ref="K88:M88"/>
     <mergeCell ref="C19:J19"/>
     <mergeCell ref="K26:M26"/>
@@ -27863,6 +28259,7 @@
     <mergeCell ref="I266:J266"/>
     <mergeCell ref="B365:F365"/>
     <mergeCell ref="I89:J89"/>
+    <mergeCell ref="F476:M476"/>
     <mergeCell ref="K96:M96"/>
     <mergeCell ref="B131:F131"/>
     <mergeCell ref="A38:M38"/>
@@ -27889,7 +28286,6 @@
     <mergeCell ref="B369:M369"/>
     <mergeCell ref="K373:M373"/>
     <mergeCell ref="I42:J42"/>
-    <mergeCell ref="A486:M486"/>
     <mergeCell ref="I284:J284"/>
     <mergeCell ref="B356:M356"/>
     <mergeCell ref="I173:J173"/>
@@ -27932,6 +28328,7 @@
     <mergeCell ref="B208:F208"/>
     <mergeCell ref="L414:M414"/>
     <mergeCell ref="K111:M111"/>
+    <mergeCell ref="F472:M472"/>
     <mergeCell ref="B82:M82"/>
     <mergeCell ref="K86:M86"/>
     <mergeCell ref="K257:M257"/>
@@ -27984,6 +28381,7 @@
     <mergeCell ref="I174:J174"/>
     <mergeCell ref="K99:M99"/>
     <mergeCell ref="C30:J30"/>
+    <mergeCell ref="A479:M479"/>
     <mergeCell ref="B136:M136"/>
     <mergeCell ref="I124:J124"/>
     <mergeCell ref="I251:J251"/>
@@ -27996,6 +28394,7 @@
     <mergeCell ref="K180:M180"/>
     <mergeCell ref="L277:M277"/>
     <mergeCell ref="I287:J287"/>
+    <mergeCell ref="A481:M481"/>
     <mergeCell ref="K130:M130"/>
     <mergeCell ref="I188:J188"/>
     <mergeCell ref="I126:J126"/>
@@ -28012,7 +28411,7 @@
     <mergeCell ref="A368:M368"/>
     <mergeCell ref="I282:J282"/>
     <mergeCell ref="K346:M346"/>
-    <mergeCell ref="E488:J488"/>
+    <mergeCell ref="F474:M474"/>
     <mergeCell ref="A36:M36"/>
     <mergeCell ref="K125:M125"/>
     <mergeCell ref="I205:J205"/>
@@ -28027,6 +28426,7 @@
     <mergeCell ref="K127:M127"/>
     <mergeCell ref="A378:M378"/>
     <mergeCell ref="I358:J358"/>
+    <mergeCell ref="F477:M477"/>
     <mergeCell ref="B93:M93"/>
     <mergeCell ref="A101:J101"/>
     <mergeCell ref="K272:M272"/>
@@ -28077,20 +28477,20 @@
     <mergeCell ref="B266:F266"/>
     <mergeCell ref="K54:M54"/>
     <mergeCell ref="B89:F89"/>
-    <mergeCell ref="E489:J489"/>
     <mergeCell ref="A50:M50"/>
     <mergeCell ref="L400:M400"/>
     <mergeCell ref="K64:M64"/>
     <mergeCell ref="B381:M381"/>
+    <mergeCell ref="E504:J504"/>
     <mergeCell ref="B97:F97"/>
     <mergeCell ref="B153:F153"/>
     <mergeCell ref="A71:J71"/>
     <mergeCell ref="B268:F268"/>
     <mergeCell ref="B324:F324"/>
     <mergeCell ref="C434:M434"/>
-    <mergeCell ref="E491:J491"/>
     <mergeCell ref="I208:J208"/>
     <mergeCell ref="K364:M364"/>
+    <mergeCell ref="E506:J506"/>
     <mergeCell ref="B170:M170"/>
     <mergeCell ref="B157:M157"/>
     <mergeCell ref="I145:J145"/>
@@ -28131,6 +28531,7 @@
     <mergeCell ref="C32:J32"/>
     <mergeCell ref="B256:F256"/>
     <mergeCell ref="K110:M110"/>
+    <mergeCell ref="A465:M465"/>
     <mergeCell ref="I69:J69"/>
     <mergeCell ref="L241:M241"/>
     <mergeCell ref="B105:M105"/>
@@ -28158,6 +28559,7 @@
     <mergeCell ref="C436:M436"/>
     <mergeCell ref="B111:F111"/>
     <mergeCell ref="K14:M14"/>
+    <mergeCell ref="E505:J505"/>
     <mergeCell ref="K207:M207"/>
     <mergeCell ref="B98:F98"/>
     <mergeCell ref="K299:M299"/>
@@ -28188,6 +28590,7 @@
     <mergeCell ref="B189:F189"/>
     <mergeCell ref="B45:F45"/>
     <mergeCell ref="K325:M325"/>
+    <mergeCell ref="F471:M471"/>
     <mergeCell ref="A242:M242"/>
     <mergeCell ref="B39:M39"/>
     <mergeCell ref="B188:F188"/>
@@ -28201,6 +28604,7 @@
     <mergeCell ref="A8:M8"/>
     <mergeCell ref="B345:F345"/>
     <mergeCell ref="K131:M131"/>
+    <mergeCell ref="F473:M473"/>
     <mergeCell ref="B193:F193"/>
     <mergeCell ref="B190:F190"/>
     <mergeCell ref="B295:F295"/>
@@ -28245,6 +28649,7 @@
     <mergeCell ref="L391:M391"/>
     <mergeCell ref="K144:M144"/>
     <mergeCell ref="B206:F206"/>
+    <mergeCell ref="A499:M499"/>
     <mergeCell ref="B203:F203"/>
     <mergeCell ref="K302:M302"/>
     <mergeCell ref="L328:M328"/>
@@ -28272,6 +28677,7 @@
     <mergeCell ref="I220:J220"/>
     <mergeCell ref="K284:M284"/>
     <mergeCell ref="K222:M222"/>
+    <mergeCell ref="E501:J501"/>
     <mergeCell ref="K234:M234"/>
     <mergeCell ref="B69:F69"/>
     <mergeCell ref="K172:M172"/>
@@ -28284,6 +28690,7 @@
     <mergeCell ref="I180:J180"/>
     <mergeCell ref="B348:F348"/>
     <mergeCell ref="L212:M212"/>
+    <mergeCell ref="E503:J503"/>
     <mergeCell ref="K236:M236"/>
     <mergeCell ref="B127:F127"/>
     <mergeCell ref="C23:J23"/>
@@ -28309,7 +28716,7 @@
     <hyperlink ref="A4" location="'14. MIMO Suggest + Incon'!A6" display="Section 1 — Suggestions"/>
     <hyperlink ref="B4" location="'14. MIMO Suggest + Incon'!A388" display="Section 2 — Dump incon"/>
     <hyperlink ref="C4" location="'14. MIMO Suggest + Incon'!A438" display="Section 3 — Final proposal"/>
-    <hyperlink ref="D4" location="'14. MIMO Suggest + Incon'!A467" display="Section 4 — Counters / KPI"/>
+    <hyperlink ref="D4" location="'14. MIMO Suggest + Incon'!A480" display="Section 4 — Counters / KPI"/>
     <hyperlink ref="A10" location="'14. MIMO Suggest + Incon'!A37" display="S15-01"/>
     <hyperlink ref="C10" location="'14. MIMO Suggest + Incon'!A37" display="Basic MIMO — PMI/SRS weight adaptation + MetaAAU beam sensing"/>
     <hyperlink ref="K10" location="'3. Step1 Basic MIMO'!A1" display="3. Step1 Basic MIMO"/>
@@ -28697,6 +29104,16 @@
     <hyperlink ref="B427" location="'14. MIMO Suggest + Incon'!A377" display="S15-25"/>
     <hyperlink ref="K427" location="'14. MIMO Suggest + Incon'!A377" display="S15-25"/>
     <hyperlink ref="L427" location="'5. Step3 MU-MIMO'!A1" display="5. Step3 MU-MIMO"/>
+    <hyperlink ref="B468" location="'14. MIMO Suggest + Incon'!A49" display="S15-02"/>
+    <hyperlink ref="B469" location="'14. MIMO Suggest + Incon'!A49" display="S15-02"/>
+    <hyperlink ref="B470" location="'14. MIMO Suggest + Incon'!A134" display="S15-09"/>
+    <hyperlink ref="B471" location="'14. MIMO Suggest + Incon'!A155" display="S15-10"/>
+    <hyperlink ref="B472" location="'14. MIMO Suggest + Incon'!A212" display="S15-14"/>
+    <hyperlink ref="B473" location="'14. MIMO Suggest + Incon'!A228" display="S15-15"/>
+    <hyperlink ref="B474" location="'14. MIMO Suggest + Incon'!A259" display="S15-17"/>
+    <hyperlink ref="B475" location="'14. MIMO Suggest + Incon'!A277" display="S15-18"/>
+    <hyperlink ref="B476" location="'14. MIMO Suggest + Incon'!A311" display="S15-20"/>
+    <hyperlink ref="B477" location="'14. MIMO Suggest + Incon'!A377" display="S15-25"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.5" header="0.25" footer="0.25"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>

</xml_diff>